<commit_message>
docs: Remove C1.3 SMS channel from Excel feature list
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Feature_List_PaymentBackoffice_02032026.xlsx
+++ b/docs/Feature_List_PaymentBackoffice_02032026.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D187"/>
+  <dimension ref="A1:D186"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="9" min="1" max="1"/>
@@ -903,108 +903,108 @@
     <row r="25" ht="15" customHeight="1" s="9">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>C1.3</t>
+          <t>C1.4</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เลือกช่องทางส่ง: Email</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="n"/>
+          <t xml:space="preserve">        กำหนดวันที่และเวลาส่ง (Scheduled Send)</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>รองรับ: ส่งทันที หรือ กำหนดเวลาล่วงหน้า</t>
+        </is>
+      </c>
       <c r="D25" s="7" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="9">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>C1.4</t>
+          <t>C1.5</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        กำหนดวันที่และเวลาส่ง (Scheduled Send)</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>รองรับ: ส่งทันที หรือ กำหนดเวลาล่วงหน้า</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ติดตามสถานะ: Draft / Scheduled / Sent / Cancelled</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="9">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>C1.5</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ติดตามสถานะ: Draft / Scheduled / Sent / Cancelled</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>C1.6</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        กรองใบแจ้งหนี้ตามวันครบกำหนด (Due Date Filter)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>แสดงเฉพาะวันที่ที่มีใบแจ้งหนี้จริงในระบบ (ตาม Academic Year / Term / Status ที่เลือก)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="9">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>C1.6</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        กรองใบแจ้งหนี้ตามวันครบกำหนด (Due Date Filter)</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>แสดงเฉพาะวันที่ที่มีใบแจ้งหนี้จริงในระบบ (ตาม Academic Year / Term / Status ที่เลือก)</t>
-        </is>
-      </c>
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    แม่แบบใบแจ้งหนี้ / ใบเสร็จ (Invoice/Receipt Template)</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1" s="9">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C2.1</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    แม่แบบใบแจ้งหนี้ / ใบเสร็จ (Invoice/Receipt Template)</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="n"/>
+          <t xml:space="preserve">        แก้ไข HTML template สำหรับอีเมลใบแจ้งหนี้และใบเสร็จ</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>รองรับ Tab แยก Edit / Preview
+ดู Live Preview ก่อนบันทึก</t>
+        </is>
+      </c>
       <c r="D29" s="7" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="9">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>C2.1</t>
+          <t>C2.2</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        แก้ไข HTML template สำหรับอีเมลใบแจ้งหนี้และใบเสร็จ</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>รองรับ Tab แยก Edit / Preview
-ดู Live Preview ก่อนบันทึก</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        บันทึกและ Reset template กลับค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="9">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>C2.2</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        บันทึกและ Reset template กลับค่าเริ่มต้น</t>
+          <t xml:space="preserve">    ประวัติการส่งอีเมล (Email History)</t>
         </is>
       </c>
       <c r="C31" s="7" t="n"/>
@@ -1013,44 +1013,44 @@
     <row r="32" ht="15" customHeight="1" s="9">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C3.1</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ประวัติการส่งอีเมล (Email History)</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="n"/>
+          <t xml:space="preserve">        ดูประวัติการส่งอีเมลทั้งหมด</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>แสดง: ผู้รับ, ประเภท, วัน-เวลา, สถานะ (Sent/Failed/Bounced)</t>
+        </is>
+      </c>
       <c r="D32" s="7" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="9">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>C3.1</t>
+          <t>C3.2</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดูประวัติการส่งอีเมลทั้งหมด</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>แสดง: ผู้รับ, ประเภท, วัน-เวลา, สถานะ (Sent/Failed/Bounced)</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ค้นหาตามผู้รับ / ประเภท / หัวข้ออีเมล</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="9">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>C3.2</t>
+          <t>C3.3</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาตามผู้รับ / ประเภท / หัวข้ออีเมล</t>
+          <t xml:space="preserve">        Export ประวัติการส่งเป็นไฟล์ Excel</t>
         </is>
       </c>
       <c r="C34" s="7" t="n"/>
@@ -1059,12 +1059,12 @@
     <row r="35" ht="15" customHeight="1" s="9">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>C3.3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Export ประวัติการส่งเป็นไฟล์ Excel</t>
+          <t xml:space="preserve">    ประวัติการชำระเงิน (Payment History)</t>
         </is>
       </c>
       <c r="C35" s="7" t="n"/>
@@ -1073,44 +1073,44 @@
     <row r="36" ht="15" customHeight="1" s="9">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C4.1</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ประวัติการชำระเงิน (Payment History)</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="n"/>
+          <t xml:space="preserve">        ดูรายการชำระเงินทั้งหมดในระบบ</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>แสดง: วันที่, นักเรียน, ยอดเงิน, วิธีชำระ, สถานะ</t>
+        </is>
+      </c>
       <c r="D36" s="7" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="9">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>C4.1</t>
+          <t>C4.2</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดูรายการชำระเงินทั้งหมดในระบบ</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>แสดง: วันที่, นักเรียน, ยอดเงิน, วิธีชำระ, สถานะ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        กรองตามวันที่ / สถานะ / นักเรียน / ยอดเงิน</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="9">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>C4.2</t>
+          <t>C4.3</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        กรองตามวันที่ / สถานะ / นักเรียน / ยอดเงิน</t>
+          <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
         </is>
       </c>
       <c r="C38" s="7" t="n"/>
@@ -1119,74 +1119,78 @@
     <row r="39" ht="15" customHeight="1" s="9">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>C4.3</t>
+          <t>C4.4</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
+          <t xml:space="preserve">        Export ข้อมูลเป็นไฟล์ Excel</t>
         </is>
       </c>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="9">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>C4.4</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Export ข้อมูลเป็นไฟล์ Excel</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>ค่าเทอม (Tuition Management)</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="9">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>ค่าเทอม (Tuition Management)</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ค่าเทอมตามปีการศึกษา (Tuition By Year)</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1" s="9">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1.1</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ค่าเทอมตามปีการศึกษา (Tuition By Year)</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="n"/>
+          <t xml:space="preserve">        แก้ไขอัตราค่าเทอมแยกตามชั้นเรียนและปีการศึกษา</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>รองรับ 16 ชั้น: Pre-Nursery ถึง Year 13
+แบ่ง 3 เทอม: Term 1, 2, 3</t>
+        </is>
+      </c>
       <c r="D42" s="7" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="9">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>D1.1</t>
+          <t>D1.2</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        แก้ไขอัตราค่าเทอมแยกตามชั้นเรียนและปีการศึกษา</t>
+          <t xml:space="preserve">        บันทึกการเปลี่ยนแปลงทั้งหมดพร้อมกัน</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>รองรับ 16 ชั้น: Pre-Nursery ถึง Year 13
-แบ่ง 3 เทอม: Term 1, 2, 3</t>
+          <t>กด Save all เพื่อบันทึกทุกชั้นพร้อมกัน</t>
         </is>
       </c>
       <c r="D43" s="7" t="n"/>
@@ -1194,30 +1198,26 @@
     <row r="44" ht="15" customHeight="1" s="9">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>D1.2</t>
+          <t>D1.3</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        บันทึกการเปลี่ยนแปลงทั้งหมดพร้อมกัน</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>กด Save all เพื่อบันทึกทุกชั้นพร้อมกัน</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        เลือกแสดงข้อมูลตามปีการศึกษา</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="n"/>
       <c r="D44" s="7" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="9">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>D1.3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เลือกแสดงข้อมูลตามปีการศึกษา</t>
+          <t xml:space="preserve">    กลุ่มส่วนลดนักเรียน (Student Discount Groups)</t>
         </is>
       </c>
       <c r="C45" s="7" t="n"/>
@@ -1226,44 +1226,44 @@
     <row r="46" ht="15" customHeight="1" s="9">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D2.1</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    กลุ่มส่วนลดนักเรียน (Student Discount Groups)</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ กลุ่มส่วนลด</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>กำหนดส่วนลดแบบ: เปอร์เซ็นต์ (%) หรือ จำนวนเงินคงที่ (Fixed Amount)</t>
+        </is>
+      </c>
       <c r="D46" s="7" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="9">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>D2.1</t>
+          <t>D2.2</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ กลุ่มส่วนลด</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>กำหนดส่วนลดแบบ: เปอร์เซ็นต์ (%) หรือ จำนวนเงินคงที่ (Fixed Amount)</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        เปิด / ปิด การใช้งานกลุ่มส่วนลด</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n"/>
       <c r="D47" s="7" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="9">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>D2.2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เปิด / ปิด การใช้งานกลุ่มส่วนลด</t>
+          <t xml:space="preserve">    จัดการใบแจ้งหนี้ค่าเทอม (Invoice Management - Tuition)</t>
         </is>
       </c>
       <c r="C48" s="7" t="n"/>
@@ -1272,44 +1272,44 @@
     <row r="49" ht="15" customHeight="1" s="9">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D3.1</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    จัดการใบแจ้งหนี้ค่าเทอม (Invoice Management - Tuition)</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="n"/>
+          <t xml:space="preserve">        ดู / เพิ่ม / แก้ไข / ลบ ใบแจ้งหนี้</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>สถานะใบแจ้งหนี้: Draft → Pending → Approved / Rejected → Sent → Paid / Overdue / Cancelled</t>
+        </is>
+      </c>
       <c r="D49" s="7" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="9">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>D3.1</t>
+          <t>D3.2</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดู / เพิ่ม / แก้ไข / ลบ ใบแจ้งหนี้</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>สถานะใบแจ้งหนี้: Draft → Pending → Approved / Rejected → Sent → Paid / Overdue / Cancelled</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ค้นหาตามเลขที่ / ชื่อนักเรียน / สถานะ / วันที่</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="n"/>
       <c r="D50" s="7" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="9">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>D3.2</t>
+          <t>D3.3</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาตามเลขที่ / ชื่อนักเรียน / สถานะ / วันที่</t>
+          <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
         </is>
       </c>
       <c r="C51" s="7" t="n"/>
@@ -1318,31 +1318,35 @@
     <row r="52" ht="15" customHeight="1" s="9">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>D3.3</t>
+          <t>D3.4</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="n"/>
+          <t xml:space="preserve">        ดำเนินการหลายรายการพร้อมกัน (Bulk Actions)</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>รองรับ: อนุมัติ, ปฏิเสธ, ทำเครื่องหมายชำระแล้ว, ส่งอีเมล, Export PDF</t>
+        </is>
+      </c>
       <c r="D52" s="7" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="9">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>D3.4</t>
+          <t>D3.5</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดำเนินการหลายรายการพร้อมกัน (Bulk Actions)</t>
+          <t xml:space="preserve">        นำเข้าข้อมูลจาก Interface File (Excel)</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>รองรับ: อนุมัติ, ปฏิเสธ, ทำเครื่องหมายชำระแล้ว, ส่งอีเมล, Export PDF</t>
+          <t>รองรับรูปแบบ Interface File สำหรับเชื่อมต่อระบบบัญชี</t>
         </is>
       </c>
       <c r="D53" s="7" t="n"/>
@@ -1350,30 +1354,26 @@
     <row r="54" ht="15" customHeight="1" s="9">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>D3.5</t>
+          <t>D3.6</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        นำเข้าข้อมูลจาก Interface File (Excel)</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="inlineStr">
-        <is>
-          <t>รองรับรูปแบบ Interface File สำหรับเชื่อมต่อระบบบัญชี</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        Export ใบแจ้งหนี้เป็น Excel / ZIP / PDF</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n"/>
       <c r="D54" s="7" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="9">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>D3.6</t>
+          <t>D3.7</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Export ใบแจ้งหนี้เป็น Excel / ZIP / PDF</t>
+          <t xml:space="preserve">        ส่งใบแจ้งหนี้ทางอีเมล พร้อมบันทึก Log</t>
         </is>
       </c>
       <c r="C55" s="7" t="n"/>
@@ -1382,63 +1382,67 @@
     <row r="56" ht="15" customHeight="1" s="9">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>D3.7</t>
+          <t>D3.8</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ส่งใบแจ้งหนี้ทางอีเมล พร้อมบันทึก Log</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="n"/>
+          <t xml:space="preserve">        สร้าง PDF ใบแจ้งหนี้</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>รวม: ข้อมูลโรงเรียน, รายการ, ส่วนลด, บัญชีธนาคาร</t>
+        </is>
+      </c>
       <c r="D56" s="7" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="9">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>D3.8</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        สร้าง PDF ใบแจ้งหนี้</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>รวม: ข้อมูลโรงเรียน, รายการ, ส่วนลด, บัญชีธนาคาร</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    รายการและแม่แบบ (Items &amp; Templates)</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="n"/>
       <c r="D57" s="7" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="9">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D4.1</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายการและแม่แบบ (Items &amp; Templates)</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ รายการค่าใช้จ่าย</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>ฟิลด์: รหัส, ชื่อ, คำอธิบาย, ยอดเงิน, หมวดหมู่, Nominal Code</t>
+        </is>
+      </c>
       <c r="D58" s="7" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="9">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>D4.1</t>
+          <t>D4.2</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ รายการค่าใช้จ่าย</t>
+          <t xml:space="preserve">        นำเข้าข้อมูลจาก Excel / CSV พร้อม Preview และตรวจสอบ Duplicate</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>ฟิลด์: รหัส, ชื่อ, คำอธิบาย, ยอดเงิน, หมวดหมู่, Nominal Code</t>
+          <t>แสดง Warning box สีเหลืองเมื่อพบรายการซ้ำ</t>
         </is>
       </c>
       <c r="D59" s="7" t="n"/>
@@ -1446,30 +1450,26 @@
     <row r="60" ht="15" customHeight="1" s="9">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>D4.2</t>
+          <t>D4.3</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        นำเข้าข้อมูลจาก Excel / CSV พร้อม Preview และตรวจสอบ Duplicate</t>
-        </is>
-      </c>
-      <c r="C60" s="7" t="inlineStr">
-        <is>
-          <t>แสดง Warning box สีเหลืองเมื่อพบรายการซ้ำ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        Export รายการทั้งหมดเป็น Excel</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n"/>
       <c r="D60" s="7" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="9">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>D4.3</t>
+          <t>D4.4</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Export รายการทั้งหมดเป็น Excel</t>
+          <t xml:space="preserve">        ค้นหาตามรหัส / ชื่อ / ชั้นเรียน และแบ่งหน้า</t>
         </is>
       </c>
       <c r="C61" s="7" t="n"/>
@@ -1478,44 +1478,44 @@
     <row r="62" ht="15" customHeight="1" s="9">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>D4.4</t>
+          <t>D4.5</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาตามรหัส / ชื่อ / ชั้นเรียน และแบ่งหน้า</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="n"/>
+          <t xml:space="preserve">        Sync ราคากับข้อมูล Tuition By Year</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>อัพเดทราคาเท่านั้น ไม่สร้างรายการใหม่อัตโนมัติ</t>
+        </is>
+      </c>
       <c r="D62" s="7" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" s="9">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>D4.5</t>
+          <t>D4.6</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Sync ราคากับข้อมูล Tuition By Year</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="inlineStr">
-        <is>
-          <t>อัพเดทราคาเท่านั้น ไม่สร้างรายการใหม่อัตโนมัติ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        เปิด / ปิด การใช้งานรายการ (Active/Inactive)</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="n"/>
       <c r="D63" s="7" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="9">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>D4.6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เปิด / ปิด การใช้งานรายการ (Active/Inactive)</t>
+          <t xml:space="preserve">    ใบเสร็จค่าเทอม (Receipts - Tuition)</t>
         </is>
       </c>
       <c r="C64" s="7" t="n"/>
@@ -1524,76 +1524,76 @@
     <row r="65" ht="15" customHeight="1" s="9">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D5.1</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบเสร็จค่าเทอม (Receipts - Tuition)</t>
-        </is>
-      </c>
-      <c r="C65" s="7" t="n"/>
+          <t xml:space="preserve">        ดูและบริหารจัดการใบเสร็จรับเงิน</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>สถานะ: Issued, Resent, Failed</t>
+        </is>
+      </c>
       <c r="D65" s="7" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="9">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>D5.1</t>
+          <t>D5.2</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดูและบริหารจัดการใบเสร็จรับเงิน</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>สถานะ: Issued, Resent, Failed</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        กรองตามสถานะ / ชั้น / เลขที่ใบเสร็จ / วันที่</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="n"/>
       <c r="D66" s="7" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="9">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>D5.2</t>
+          <t>D5.3</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        กรองตามสถานะ / ชั้น / เลขที่ใบเสร็จ / วันที่</t>
-        </is>
-      </c>
-      <c r="C67" s="7" t="n"/>
+          <t xml:space="preserve">        ดำเนินการหลายรายการพร้อมกัน (Bulk Actions)</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>รองรับ: อนุมัติ, แก้ไข, ลบ</t>
+        </is>
+      </c>
       <c r="D67" s="7" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="9">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>D5.3</t>
+          <t>D5.4</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดำเนินการหลายรายการพร้อมกัน (Bulk Actions)</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>รองรับ: อนุมัติ, แก้ไข, ลบ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        สร้าง PDF ใบเสร็จรับเงิน</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n"/>
       <c r="D68" s="7" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="9">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>D5.4</t>
+          <t>D5.5</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        สร้าง PDF ใบเสร็จรับเงิน</t>
+          <t xml:space="preserve">        นำเข้าและ Export ข้อมูลใบเสร็จ</t>
         </is>
       </c>
       <c r="C69" s="7" t="n"/>
@@ -1602,12 +1602,12 @@
     <row r="70" ht="15" customHeight="1" s="9">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>D5.5</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        นำเข้าและ Export ข้อมูลใบเสร็จ</t>
+          <t xml:space="preserve">    ใบลดหนี้ (Credit Notes)</t>
         </is>
       </c>
       <c r="C70" s="7" t="n"/>
@@ -1616,151 +1616,151 @@
     <row r="71" ht="30" customHeight="1" s="9">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D6.1</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบลดหนี้ (Credit Notes)</t>
-        </is>
-      </c>
-      <c r="C71" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ใบลดหนี้</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>ประเภท: Refund, Adjustment, Cancellation
+สถานะ: Draft, Issued, Applied, Cancelled</t>
+        </is>
+      </c>
       <c r="D71" s="7" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="9">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>D6.1</t>
+          <t>D6.2</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ใบลดหนี้</t>
-        </is>
-      </c>
-      <c r="C72" s="7" t="inlineStr">
-        <is>
-          <t>ประเภท: Refund, Adjustment, Cancellation
-สถานะ: Draft, Issued, Applied, Cancelled</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ค้นหาตามเลขที่ / ชื่อนักเรียน / สถานะ และแบ่งหน้า</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="n"/>
       <c r="D72" s="7" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="9">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>D6.2</t>
+          <t>D6.3</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาตามเลขที่ / ชื่อนักเรียน / สถานะ และแบ่งหน้า</t>
+          <t xml:space="preserve">        นำเข้าและ Export ข้อมูลใบลดหนี้เป็น Excel</t>
         </is>
       </c>
       <c r="C73" s="7" t="n"/>
       <c r="D73" s="7" t="n"/>
     </row>
     <row r="74" ht="18" customHeight="1" s="9">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>D6.3</t>
-        </is>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        นำเข้าและ Export ข้อมูลใบลดหนี้เป็น Excel</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="n"/>
-      <c r="D74" s="7" t="n"/>
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>กิจกรรมนอกเวลา (ECA / After School)</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="n"/>
+      <c r="D74" s="6" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" s="9">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>กิจกรรมนอกเวลา (ECA / After School)</t>
-        </is>
-      </c>
-      <c r="C75" s="6" t="n"/>
-      <c r="D75" s="6" t="n"/>
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ใบแจ้งหนี้ ECA</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="n"/>
+      <c r="D75" s="7" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" s="9">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>E1.1</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบแจ้งหนี้ ECA</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>หมวดหมู่: ECA (เช่น ดนตรี, กีฬา, ชมรม)</t>
+        </is>
+      </c>
       <c r="D76" s="7" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" s="9">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>E1.1</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
-        </is>
-      </c>
-      <c r="C77" s="7" t="inlineStr">
-        <is>
-          <t>หมวดหมู่: ECA (เช่น ดนตรี, กีฬา, ชมรม)</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    รายการและแม่แบบ ECA</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="n"/>
       <c r="D77" s="7" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" s="9">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E2.1</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายการและแม่แบบ ECA</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>มีตัวอย่างรายการ: Piano, Guitar, Violin ฯลฯ</t>
+        </is>
+      </c>
       <c r="D78" s="7" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1" s="9">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>E2.1</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
-        </is>
-      </c>
-      <c r="C79" s="7" t="inlineStr">
-        <is>
-          <t>มีตัวอย่างรายการ: Piano, Guitar, Violin ฯลฯ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    ใบเสร็จ ECA</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="n"/>
       <c r="D79" s="7" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="9">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E3.1</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบเสร็จ ECA</t>
+          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
       <c r="C80" s="7" t="n"/>
@@ -1769,12 +1769,12 @@
     <row r="81" ht="15" customHeight="1" s="9">
       <c r="A81" s="7" t="inlineStr">
         <is>
-          <t>E3.1</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
+          <t xml:space="preserve">    กลุ่มส่วนลด ECA</t>
         </is>
       </c>
       <c r="C81" s="7" t="n"/>
@@ -1783,86 +1783,86 @@
     <row r="82" ht="15" customHeight="1" s="9">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E4.1</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    กลุ่มส่วนลด ECA</t>
+          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด ECA</t>
         </is>
       </c>
       <c r="C82" s="7" t="n"/>
       <c r="D82" s="7" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1" s="9">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>E4.1</t>
-        </is>
-      </c>
-      <c r="B83" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด ECA</t>
-        </is>
-      </c>
-      <c r="C83" s="7" t="n"/>
-      <c r="D83" s="7" t="n"/>
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>ทริปและกิจกรรม (Trip &amp; Activity)</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1" s="9">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>ทริปและกิจกรรม (Trip &amp; Activity)</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="n"/>
-      <c r="D84" s="6" t="n"/>
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ใบแจ้งหนี้ทริป</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="n"/>
+      <c r="D84" s="7" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="9">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1.1</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบแจ้งหนี้ทริป</t>
-        </is>
-      </c>
-      <c r="C85" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>หมวดหมู่: trip</t>
+        </is>
+      </c>
       <c r="D85" s="7" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="9">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>F1.1</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
-        </is>
-      </c>
-      <c r="C86" s="7" t="inlineStr">
-        <is>
-          <t>หมวดหมู่: trip</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    รายการและแม่แบบทริป</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="n"/>
       <c r="D86" s="7" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="9">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F2.1</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายการและแม่แบบทริป</t>
+          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
         </is>
       </c>
       <c r="C87" s="7" t="n"/>
@@ -1871,12 +1871,12 @@
     <row r="88" ht="15" customHeight="1" s="9">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>F2.1</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
+          <t xml:space="preserve">    ใบเสร็จทริป</t>
         </is>
       </c>
       <c r="C88" s="7" t="n"/>
@@ -1885,12 +1885,12 @@
     <row r="89" ht="15" customHeight="1" s="9">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F3.1</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบเสร็จทริป</t>
+          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
       <c r="C89" s="7" t="n"/>
@@ -1899,12 +1899,12 @@
     <row r="90" ht="15" customHeight="1" s="9">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>F3.1</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
+          <t xml:space="preserve">    กลุ่มส่วนลดทริป</t>
         </is>
       </c>
       <c r="C90" s="7" t="n"/>
@@ -1913,86 +1913,86 @@
     <row r="91" ht="15" customHeight="1" s="9">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F4.1</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    กลุ่มส่วนลดทริป</t>
+          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Trip</t>
         </is>
       </c>
       <c r="C91" s="7" t="n"/>
       <c r="D91" s="7" t="n"/>
     </row>
     <row r="92" ht="18" customHeight="1" s="9">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t>F4.1</t>
-        </is>
-      </c>
-      <c r="B92" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Trip</t>
-        </is>
-      </c>
-      <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="n"/>
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>ค่าสอบ (Exam)</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="n"/>
+      <c r="D92" s="6" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="9">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>ค่าสอบ (Exam)</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="n"/>
-      <c r="D93" s="6" t="n"/>
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ใบแจ้งหนี้ค่าสอบ</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="n"/>
+      <c r="D93" s="7" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="9">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G1.1</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบแจ้งหนี้ค่าสอบ</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>หมวดหมู่: exam</t>
+        </is>
+      </c>
       <c r="D94" s="7" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="9">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>G1.1</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
-        </is>
-      </c>
-      <c r="C95" s="7" t="inlineStr">
-        <is>
-          <t>หมวดหมู่: exam</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    รายการและแม่แบบค่าสอบ</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="n"/>
       <c r="D95" s="7" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1" s="9">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G2.1</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายการและแม่แบบค่าสอบ</t>
+          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
         </is>
       </c>
       <c r="C96" s="7" t="n"/>
@@ -2001,12 +2001,12 @@
     <row r="97" ht="15" customHeight="1" s="9">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t>G2.1</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
+          <t xml:space="preserve">    ใบเสร็จค่าสอบ</t>
         </is>
       </c>
       <c r="C97" s="7" t="n"/>
@@ -2015,12 +2015,12 @@
     <row r="98" ht="15" customHeight="1" s="9">
       <c r="A98" s="7" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G3.1</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบเสร็จค่าสอบ</t>
+          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
       <c r="C98" s="7" t="n"/>
@@ -2029,12 +2029,12 @@
     <row r="99" ht="15" customHeight="1" s="9">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>G3.1</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
+          <t xml:space="preserve">    กลุ่มส่วนลดค่าสอบ</t>
         </is>
       </c>
       <c r="C99" s="7" t="n"/>
@@ -2043,118 +2043,118 @@
     <row r="100" ht="15" customHeight="1" s="9">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>G4.1</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    กลุ่มส่วนลดค่าสอบ</t>
+          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Exam</t>
         </is>
       </c>
       <c r="C100" s="7" t="n"/>
       <c r="D100" s="7" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1" s="9">
-      <c r="A101" s="7" t="inlineStr">
-        <is>
-          <t>G4.1</t>
-        </is>
-      </c>
-      <c r="B101" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Exam</t>
-        </is>
-      </c>
-      <c r="C101" s="7" t="n"/>
-      <c r="D101" s="7" t="n"/>
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>รถรับส่ง (School Bus)</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1" s="9">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B102" s="6" t="inlineStr">
-        <is>
-          <t>รถรับส่ง (School Bus)</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="n"/>
-      <c r="D102" s="6" t="n"/>
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ใบแจ้งหนี้รถรับส่ง</t>
+        </is>
+      </c>
+      <c r="C102" s="7" t="n"/>
+      <c r="D102" s="7" t="n"/>
     </row>
     <row r="103" ht="15" customHeight="1" s="9">
       <c r="A103" s="7" t="inlineStr">
         <is>
-          <t>H1</t>
+          <t>H1.1</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบแจ้งหนี้รถรับส่ง</t>
-        </is>
-      </c>
-      <c r="C103" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>หมวดหมู่: bus</t>
+        </is>
+      </c>
       <c r="D103" s="7" t="n"/>
     </row>
     <row r="104" ht="15" customHeight="1" s="9">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>H1.1</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
-        </is>
-      </c>
-      <c r="C104" s="7" t="inlineStr">
-        <is>
-          <t>หมวดหมู่: bus</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    รายการและแม่แบบรถรับส่ง</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="n"/>
       <c r="D104" s="7" t="n"/>
     </row>
     <row r="105" ht="15" customHeight="1" s="9">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>H2.1</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายการและแม่แบบรถรับส่ง</t>
-        </is>
-      </c>
-      <c r="C105" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>รายการตามเส้นทาง/จุดรับส่ง</t>
+        </is>
+      </c>
       <c r="D105" s="7" t="n"/>
     </row>
     <row r="106" ht="15" customHeight="1" s="9">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>H2.1</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
-        </is>
-      </c>
-      <c r="C106" s="7" t="inlineStr">
-        <is>
-          <t>รายการตามเส้นทาง/จุดรับส่ง</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    ใบเสร็จรถรับส่ง</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="n"/>
       <c r="D106" s="7" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="9">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t>H3</t>
+          <t>H3.1</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบเสร็จรถรับส่ง</t>
+          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
       <c r="C107" s="7" t="n"/>
@@ -2163,12 +2163,12 @@
     <row r="108" ht="15" customHeight="1" s="9">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>H3.1</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
+          <t xml:space="preserve">    กลุ่มส่วนลดรถรับส่ง</t>
         </is>
       </c>
       <c r="C108" s="7" t="n"/>
@@ -2177,74 +2177,78 @@
     <row r="109" ht="15" customHeight="1" s="9">
       <c r="A109" s="7" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>H4.1</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    กลุ่มส่วนลดรถรับส่ง</t>
+          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Bus</t>
         </is>
       </c>
       <c r="C109" s="7" t="n"/>
       <c r="D109" s="7" t="n"/>
     </row>
     <row r="110" ht="18" customHeight="1" s="9">
-      <c r="A110" s="7" t="inlineStr">
-        <is>
-          <t>H4.1</t>
-        </is>
-      </c>
-      <c r="B110" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Bus</t>
-        </is>
-      </c>
-      <c r="C110" s="7" t="n"/>
-      <c r="D110" s="7" t="n"/>
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>ใบแจ้งหนี้บุคคลภายนอก (External Invoice)</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="n"/>
+      <c r="D110" s="6" t="n"/>
     </row>
     <row r="111" ht="15" customHeight="1" s="9">
-      <c r="A111" s="6" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B111" s="6" t="inlineStr">
-        <is>
-          <t>ใบแจ้งหนี้บุคคลภายนอก (External Invoice)</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="n"/>
-      <c r="D111" s="6" t="n"/>
+      <c r="A111" s="7" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ใบแจ้งหนี้ภายนอก</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="n"/>
+      <c r="D111" s="7" t="n"/>
     </row>
     <row r="112" ht="30" customHeight="1" s="9">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>I1</t>
+          <t>I1.1</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบแจ้งหนี้ภายนอก</t>
-        </is>
-      </c>
-      <c r="C112" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>หมวดหมู่: external
+ผู้รับ: บุคคล/องค์กรภายนอก (ไม่ใช่นักเรียน)</t>
+        </is>
+      </c>
       <c r="D112" s="7" t="n"/>
     </row>
     <row r="113" ht="15" customHeight="1" s="9">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t>I1.1</t>
+          <t>I1.2</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Bulk Actions, Export, Email, PDF — เหมือน Tuition Invoice</t>
+          <t xml:space="preserve">        สร้างใบแจ้งหนี้สำหรับลูกค้าภายนอก</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>หมวดหมู่: external
-ผู้รับ: บุคคล/องค์กรภายนอก (ไม่ใช่นักเรียน)</t>
+          <t>ระบุ: ชื่อผู้รับ, ที่อยู่, อีเมล, ชื่องาน</t>
         </is>
       </c>
       <c r="D113" s="7" t="n"/>
@@ -2252,82 +2256,82 @@
     <row r="114" ht="15" customHeight="1" s="9">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t>I1.2</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        สร้างใบแจ้งหนี้สำหรับลูกค้าภายนอก</t>
-        </is>
-      </c>
-      <c r="C114" s="7" t="inlineStr">
-        <is>
-          <t>ระบุ: ชื่อผู้รับ, ที่อยู่, อีเมล, ชื่องาน</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    รายชื่อลูกค้า (Client List)</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="n"/>
       <c r="D114" s="7" t="n"/>
     </row>
     <row r="115" ht="15" customHeight="1" s="9">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>I2.1</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายชื่อลูกค้า (Client List)</t>
-        </is>
-      </c>
-      <c r="C115" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ข้อมูลลูกค้า</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>ฟิลด์: ชื่อบริษัท/บุคคล, ชื่อผู้ติดต่อ, ที่อยู่</t>
+        </is>
+      </c>
       <c r="D115" s="7" t="n"/>
     </row>
     <row r="116" ht="15" customHeight="1" s="9">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>I2.1</t>
+          <t>I2.2</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ข้อมูลลูกค้า</t>
-        </is>
-      </c>
-      <c r="C116" s="7" t="inlineStr">
-        <is>
-          <t>ฟิลด์: ชื่อบริษัท/บุคคล, ชื่อผู้ติดต่อ, ที่อยู่</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ค้นหาลูกค้า</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="n"/>
       <c r="D116" s="7" t="n"/>
     </row>
     <row r="117" ht="30" customHeight="1" s="9">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>I2.2</t>
+          <t>I2.3</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาลูกค้า</t>
-        </is>
-      </c>
-      <c r="C117" s="7" t="n"/>
+          <t xml:space="preserve">        นำเข้าลูกค้าจาก Excel / CSV</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>Column ที่ต้องการ: Client Name (required), Contact Name, Address
+รองรับ Preview และตรวจสอบ Duplicate</t>
+        </is>
+      </c>
       <c r="D117" s="7" t="n"/>
     </row>
     <row r="118" ht="15" customHeight="1" s="9">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>I2.3</t>
+          <t>I2.4</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        นำเข้าลูกค้าจาก Excel / CSV</t>
+          <t xml:space="preserve">        Export รายชื่อลูกค้าเป็น Excel</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>Column ที่ต้องการ: Client Name (required), Contact Name, Address
-รองรับ Preview และตรวจสอบ Duplicate</t>
+          <t>Export ตามรายการที่ filter อยู่ปัจจุบัน</t>
         </is>
       </c>
       <c r="D118" s="7" t="n"/>
@@ -2335,62 +2339,58 @@
     <row r="119" ht="15" customHeight="1" s="9">
       <c r="A119" s="7" t="inlineStr">
         <is>
-          <t>I2.4</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Export รายชื่อลูกค้าเป็น Excel</t>
-        </is>
-      </c>
-      <c r="C119" s="7" t="inlineStr">
-        <is>
-          <t>Export ตามรายการที่ filter อยู่ปัจจุบัน</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    รายการและแม่แบบภายนอก</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="n"/>
       <c r="D119" s="7" t="n"/>
     </row>
     <row r="120" ht="15" customHeight="1" s="9">
       <c r="A120" s="7" t="inlineStr">
         <is>
-          <t>I3</t>
+          <t>I3.1</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายการและแม่แบบภายนอก</t>
-        </is>
-      </c>
-      <c r="C120" s="7" t="n"/>
+          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>ประเภท: Rental, Catering, Service, Event, Other</t>
+        </is>
+      </c>
       <c r="D120" s="7" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1" s="9">
       <c r="A121" s="7" t="inlineStr">
         <is>
-          <t>I3.1</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
-        </is>
-      </c>
-      <c r="C121" s="7" t="inlineStr">
-        <is>
-          <t>ประเภท: Rental, Catering, Service, Event, Other</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    ใบเสร็จภายนอก</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="n"/>
       <c r="D121" s="7" t="n"/>
     </row>
     <row r="122" ht="15" customHeight="1" s="9">
       <c r="A122" s="7" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>I4.1</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ใบเสร็จภายนอก</t>
+          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
       <c r="C122" s="7" t="n"/>
@@ -2399,12 +2399,12 @@
     <row r="123" ht="15" customHeight="1" s="9">
       <c r="A123" s="7" t="inlineStr">
         <is>
-          <t>I4.1</t>
+          <t>I5</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
+          <t xml:space="preserve">    กลุ่มส่วนลดภายนอก</t>
         </is>
       </c>
       <c r="C123" s="7" t="n"/>
@@ -2413,86 +2413,86 @@
     <row r="124" ht="15" customHeight="1" s="9">
       <c r="A124" s="7" t="inlineStr">
         <is>
-          <t>I5</t>
+          <t>I5.1</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    กลุ่มส่วนลดภายนอก</t>
+          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด External</t>
         </is>
       </c>
       <c r="C124" s="7" t="n"/>
       <c r="D124" s="7" t="n"/>
     </row>
     <row r="125" ht="18" customHeight="1" s="9">
-      <c r="A125" s="7" t="inlineStr">
-        <is>
-          <t>I5.1</t>
-        </is>
-      </c>
-      <c r="B125" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด External</t>
-        </is>
-      </c>
-      <c r="C125" s="7" t="n"/>
-      <c r="D125" s="7" t="n"/>
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>ข้อมูลนักเรียน (Student Management)</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="n"/>
+      <c r="D125" s="6" t="n"/>
     </row>
     <row r="126" ht="15" customHeight="1" s="9">
-      <c r="A126" s="6" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>ข้อมูลนักเรียน (Student Management)</t>
-        </is>
-      </c>
-      <c r="C126" s="6" t="n"/>
-      <c r="D126" s="6" t="n"/>
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t>J1</t>
+        </is>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    รายชื่อนักเรียน (Student List)</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="n"/>
+      <c r="D126" s="7" t="n"/>
     </row>
     <row r="127" ht="15" customHeight="1" s="9">
       <c r="A127" s="7" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J1.1</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายชื่อนักเรียน (Student List)</t>
-        </is>
-      </c>
-      <c r="C127" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ข้อมูลนักเรียน</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t>ฟิลด์: ชื่อ, รหัส, ชั้น, วันเกิด, เพศ, สถานะ, ปีการศึกษา, ครอบครัว, ผู้ปกครอง</t>
+        </is>
+      </c>
       <c r="D127" s="7" t="n"/>
     </row>
     <row r="128" ht="15" customHeight="1" s="9">
       <c r="A128" s="7" t="inlineStr">
         <is>
-          <t>J1.1</t>
+          <t>J1.2</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ข้อมูลนักเรียน</t>
-        </is>
-      </c>
-      <c r="C128" s="7" t="inlineStr">
-        <is>
-          <t>ฟิลด์: ชื่อ, รหัส, ชั้น, วันเกิด, เพศ, สถานะ, ปีการศึกษา, ครอบครัว, ผู้ปกครอง</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ค้นหาตามชื่อ / รหัส และกรองตามสถานะ / ชั้น / ปีการศึกษา / เทอม</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="n"/>
       <c r="D128" s="7" t="n"/>
     </row>
     <row r="129" ht="15" customHeight="1" s="9">
       <c r="A129" s="7" t="inlineStr">
         <is>
-          <t>J1.2</t>
+          <t>J1.3</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาตามชื่อ / รหัส และกรองตามสถานะ / ชั้น / ปีการศึกษา / เทอม</t>
+          <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
         </is>
       </c>
       <c r="C129" s="7" t="n"/>
@@ -2501,188 +2501,188 @@
     <row r="130" ht="30" customHeight="1" s="9">
       <c r="A130" s="7" t="inlineStr">
         <is>
-          <t>J1.3</t>
+          <t>J1.4</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
-        </is>
-      </c>
-      <c r="C130" s="7" t="n"/>
+          <t xml:space="preserve">        นำเข้านักเรียนจาก Excel / CSV</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>Column ที่ต้องการ: Student ID, First Name (หรือ Name), Year Group, Academic Year (หรือ Year)
+แสดง Preview 10 แถวแรก + Toggle แสดงทั้งหมด</t>
+        </is>
+      </c>
       <c r="D130" s="7" t="n"/>
     </row>
     <row r="131" ht="15" customHeight="1" s="9">
       <c r="A131" s="7" t="inlineStr">
         <is>
-          <t>J1.4</t>
+          <t>J1.5</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        นำเข้านักเรียนจาก Excel / CSV</t>
+          <t xml:space="preserve">        Export รายชื่อนักเรียนเป็น Excel (25 columns)</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>Column ที่ต้องการ: Student ID, First Name (หรือ Name), Year Group, Academic Year (หรือ Year)
-แสดง Preview 10 แถวแรก + Toggle แสดงทั้งหมด</t>
+          <t>รวม: ข้อมูลส่วนตัว, ครอบครัว, ผู้ปกครอง 2 คน, วันลงทะเบียน</t>
         </is>
       </c>
       <c r="D131" s="7" t="n"/>
     </row>
     <row r="132" ht="15" customHeight="1" s="9">
-      <c r="A132" s="7" t="inlineStr">
-        <is>
-          <t>J1.5</t>
-        </is>
-      </c>
-      <c r="B132" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Export รายชื่อนักเรียนเป็น Excel (25 columns)</t>
-        </is>
-      </c>
-      <c r="C132" s="7" t="inlineStr">
-        <is>
-          <t>รวม: ข้อมูลส่วนตัว, ครอบครัว, ผู้ปกครอง 2 คน, วันลงทะเบียน</t>
-        </is>
-      </c>
-      <c r="D132" s="7" t="n"/>
-    </row>
-    <row r="133" ht="30" customHeight="1" s="9">
-      <c r="A133" t="inlineStr">
+      <c r="A132" t="inlineStr">
         <is>
           <t>J1.6</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B132" t="inlineStr">
         <is>
           <t xml:space="preserve">        แสดง Term จากใบแจ้งหนี้จริง (ไม่ใช่ Enrollment Term)</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>Term column แสดงทุกเทอมที่นักเรียนมีใบแจ้งหนี้ เช่น Term 1 · Term 2
 Filter Term กรองตาม invoice จริง</t>
         </is>
       </c>
     </row>
+    <row r="133" ht="30" customHeight="1" s="9">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    กลุ่มครอบครัว (Family Groups)</t>
+        </is>
+      </c>
+      <c r="C133" s="7" t="n"/>
+      <c r="D133" s="7" t="n"/>
+    </row>
     <row r="134" ht="15" customHeight="1" s="9">
       <c r="A134" s="7" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J2.1</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    กลุ่มครอบครัว (Family Groups)</t>
-        </is>
-      </c>
-      <c r="C134" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ข้อมูลครอบครัว</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t>รองรับหลายบุตรต่อครอบครัว
+ฟิลด์: Family Code, ชื่อครอบครัว, ที่อยู่, Email สำหรับใบแจ้งหนี้</t>
+        </is>
+      </c>
       <c r="D134" s="7" t="n"/>
     </row>
     <row r="135" ht="15" customHeight="1" s="9">
       <c r="A135" s="7" t="inlineStr">
         <is>
-          <t>J2.1</t>
+          <t>J2.2</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ข้อมูลครอบครัว</t>
-        </is>
-      </c>
-      <c r="C135" s="7" t="inlineStr">
-        <is>
-          <t>รองรับหลายบุตรต่อครอบครัว
-ฟิลด์: Family Code, ชื่อครอบครัว, ที่อยู่, Email สำหรับใบแจ้งหนี้</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ค้นหาและกรองข้อมูลครอบครัว และแบ่งหน้า</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="n"/>
       <c r="D135" s="7" t="n"/>
     </row>
     <row r="136" ht="18" customHeight="1" s="9">
       <c r="A136" s="7" t="inlineStr">
         <is>
-          <t>J2.2</t>
+          <t>J2.3</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาและกรองข้อมูลครอบครัว และแบ่งหน้า</t>
+          <t xml:space="preserve">        Export ข้อมูลครอบครัวเป็น Excel</t>
         </is>
       </c>
       <c r="C136" s="7" t="n"/>
       <c r="D136" s="7" t="n"/>
     </row>
     <row r="137" ht="15" customHeight="1" s="9">
-      <c r="A137" s="7" t="inlineStr">
-        <is>
-          <t>J2.3</t>
-        </is>
-      </c>
-      <c r="B137" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Export ข้อมูลครอบครัวเป็น Excel</t>
-        </is>
-      </c>
-      <c r="C137" s="7" t="n"/>
-      <c r="D137" s="7" t="n"/>
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B137" s="6" t="inlineStr">
+        <is>
+          <t>การจัดการส่วนลด (Discount Management)</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="n"/>
+      <c r="D137" s="6" t="n"/>
     </row>
     <row r="138" ht="15" customHeight="1" s="9">
-      <c r="A138" s="6" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="B138" s="6" t="inlineStr">
-        <is>
-          <t>การจัดการส่วนลด (Discount Management)</t>
-        </is>
-      </c>
-      <c r="C138" s="6" t="n"/>
-      <c r="D138" s="6" t="n"/>
+      <c r="A138" s="7" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    โปรโมชั่น (Promotional Campaigns)</t>
+        </is>
+      </c>
+      <c r="C138" s="7" t="n"/>
+      <c r="D138" s="7" t="n"/>
     </row>
     <row r="139" ht="15" customHeight="1" s="9">
       <c r="A139" s="7" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K1.1</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    โปรโมชั่น (Promotional Campaigns)</t>
-        </is>
-      </c>
-      <c r="C139" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ โปรโมชั่น [ถูกลบออกจากระบบ]</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t>กำหนด: ชื่อ, ประเภทส่วนลด (% หรือ Fixed), วันเริ่ม-สิ้นสุด, สถานะ</t>
+        </is>
+      </c>
       <c r="D139" s="7" t="n"/>
     </row>
     <row r="140" ht="15" customHeight="1" s="9">
       <c r="A140" s="7" t="inlineStr">
         <is>
-          <t>K1.1</t>
+          <t>K1.2</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ โปรโมชั่น [ถูกลบออกจากระบบ]</t>
-        </is>
-      </c>
-      <c r="C140" s="7" t="inlineStr">
-        <is>
-          <t>กำหนด: ชื่อ, ประเภทส่วนลด (% หรือ Fixed), วันเริ่ม-สิ้นสุด, สถานะ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ติดตามสถานะ: Active / Ended / Scheduled [ถูกลบออกจากระบบ]</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="n"/>
       <c r="D140" s="7" t="n"/>
     </row>
     <row r="141" ht="15" customHeight="1" s="9">
       <c r="A141" s="7" t="inlineStr">
         <is>
-          <t>K1.2</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ติดตามสถานะ: Active / Ended / Scheduled [ถูกลบออกจากระบบ]</t>
+          <t xml:space="preserve">    จัดการยกเว้นค่าเทอม (Waive Fee Management)</t>
         </is>
       </c>
       <c r="C141" s="7" t="n"/>
@@ -2691,44 +2691,44 @@
     <row r="142" ht="15" customHeight="1" s="9">
       <c r="A142" s="7" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K2.1</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    จัดการยกเว้นค่าเทอม (Waive Fee Management)</t>
-        </is>
-      </c>
-      <c r="C142" s="7" t="n"/>
+          <t xml:space="preserve">        ดูรายชื่อนักเรียนที่มีสิทธิ์ยกเว้นค่าเทอม</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>ประเภท: Sibling Discount, Staff Child, Scholarship, Early Bird</t>
+        </is>
+      </c>
       <c r="D142" s="7" t="n"/>
     </row>
     <row r="143" ht="15" customHeight="1" s="9">
       <c r="A143" s="7" t="inlineStr">
         <is>
-          <t>K2.1</t>
+          <t>K2.2</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดูรายชื่อนักเรียนที่มีสิทธิ์ยกเว้นค่าเทอม</t>
-        </is>
-      </c>
-      <c r="C143" s="7" t="inlineStr">
-        <is>
-          <t>ประเภท: Sibling Discount, Staff Child, Scholarship, Early Bird</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        กรองตามสถานะและปีการศึกษา</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="n"/>
       <c r="D143" s="7" t="n"/>
     </row>
     <row r="144" ht="15" customHeight="1" s="9">
       <c r="A144" s="7" t="inlineStr">
         <is>
-          <t>K2.2</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        กรองตามสถานะและปีการศึกษา</t>
+          <t xml:space="preserve">    รายละเอียดยกเว้นรายปี (Waive Fee Year Details)</t>
         </is>
       </c>
       <c r="C144" s="7" t="n"/>
@@ -2737,78 +2737,82 @@
     <row r="145" ht="18" customHeight="1" s="9">
       <c r="A145" s="7" t="inlineStr">
         <is>
-          <t>K3</t>
+          <t>K3.1</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    รายละเอียดยกเว้นรายปี (Waive Fee Year Details)</t>
-        </is>
-      </c>
-      <c r="C145" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข รายการยกเว้นค่าเทอมรายปี</t>
+        </is>
+      </c>
+      <c r="C145" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหาตามชื่อนักเรียน / สถานะ</t>
+        </is>
+      </c>
       <c r="D145" s="7" t="n"/>
     </row>
     <row r="146" ht="15" customHeight="1" s="9">
-      <c r="A146" s="7" t="inlineStr">
-        <is>
-          <t>K3.1</t>
-        </is>
-      </c>
-      <c r="B146" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข รายการยกเว้นค่าเทอมรายปี</t>
-        </is>
-      </c>
-      <c r="C146" s="7" t="inlineStr">
-        <is>
-          <t>ค้นหาตามชื่อนักเรียน / สถานะ</t>
-        </is>
-      </c>
-      <c r="D146" s="7" t="n"/>
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>การอนุมัติและสร้างใบแจ้งหนี้ (Approval &amp; Invoice Creation)</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="n"/>
+      <c r="D146" s="6" t="n"/>
     </row>
     <row r="147" ht="30" customHeight="1" s="9">
-      <c r="A147" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="B147" s="6" t="inlineStr">
-        <is>
-          <t>การอนุมัติและสร้างใบแจ้งหนี้ (Approval &amp; Invoice Creation)</t>
-        </is>
-      </c>
-      <c r="C147" s="6" t="n"/>
-      <c r="D147" s="6" t="n"/>
+      <c r="A147" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    คิวอนุมัติ (Approval Queue)</t>
+        </is>
+      </c>
+      <c r="C147" s="7" t="n"/>
+      <c r="D147" s="7" t="n"/>
     </row>
     <row r="148" ht="15" customHeight="1" s="9">
       <c r="A148" s="7" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L1.1</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    คิวอนุมัติ (Approval Queue)</t>
-        </is>
-      </c>
-      <c r="C148" s="7" t="n"/>
+          <t xml:space="preserve">        ดูรายการใบแจ้งหนี้ที่รออนุมัติ</t>
+        </is>
+      </c>
+      <c r="C148" s="7" t="inlineStr">
+        <is>
+          <t>แสดงสถานะ: Wait / Approved / Rejected
+เลขที่ใบแจ้งหนี้แสดงเฉพาะ Approved</t>
+        </is>
+      </c>
       <c r="D148" s="7" t="n"/>
     </row>
     <row r="149" ht="15" customHeight="1" s="9">
       <c r="A149" s="7" t="inlineStr">
         <is>
-          <t>L1.1</t>
+          <t>L1.2</t>
         </is>
       </c>
       <c r="B149" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดูรายการใบแจ้งหนี้ที่รออนุมัติ</t>
+          <t xml:space="preserve">        อนุมัติหรือปฏิเสธใบแจ้งหนี้ พร้อมระบุเหตุผล</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>แสดงสถานะ: Wait / Approved / Rejected
-เลขที่ใบแจ้งหนี้แสดงเฉพาะ Approved</t>
+          <t>บันทึก: Approved by, Approved at, Rejected reason</t>
         </is>
       </c>
       <c r="D149" s="7" t="n"/>
@@ -2816,30 +2820,26 @@
     <row r="150" ht="15" customHeight="1" s="9">
       <c r="A150" s="7" t="inlineStr">
         <is>
-          <t>L1.2</t>
+          <t>L1.3</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        อนุมัติหรือปฏิเสธใบแจ้งหนี้ พร้อมระบุเหตุผล</t>
-        </is>
-      </c>
-      <c r="C150" s="7" t="inlineStr">
-        <is>
-          <t>บันทึก: Approved by, Approved at, Rejected reason</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        กรองตามสถานะ / วันที่ / ชื่อนักเรียน และแบ่งหน้า</t>
+        </is>
+      </c>
+      <c r="C150" s="7" t="n"/>
       <c r="D150" s="7" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1" s="9">
       <c r="A151" s="7" t="inlineStr">
         <is>
-          <t>L1.3</t>
+          <t>L1.4</t>
         </is>
       </c>
       <c r="B151" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        กรองตามสถานะ / วันที่ / ชื่อนักเรียน และแบ่งหน้า</t>
+          <t xml:space="preserve">        ดำเนินการหลายรายการพร้อมกัน (Bulk Approve)</t>
         </is>
       </c>
       <c r="C151" s="7" t="n"/>
@@ -2848,12 +2848,12 @@
     <row r="152" ht="15" customHeight="1" s="9">
       <c r="A152" s="7" t="inlineStr">
         <is>
-          <t>L1.4</t>
+          <t>L1.5</t>
         </is>
       </c>
       <c r="B152" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดำเนินการหลายรายการพร้อมกัน (Bulk Approve)</t>
+          <t xml:space="preserve">        Export ใบแจ้งหนี้เป็น Excel / PDF</t>
         </is>
       </c>
       <c r="C152" s="7" t="n"/>
@@ -2862,12 +2862,12 @@
     <row r="153" ht="15" customHeight="1" s="9">
       <c r="A153" s="7" t="inlineStr">
         <is>
-          <t>L1.5</t>
+          <t>L1.6</t>
         </is>
       </c>
       <c r="B153" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Export ใบแจ้งหนี้เป็น Excel / PDF</t>
+          <t xml:space="preserve">        ส่งอีเมลแจ้งผลการอนุมัติ</t>
         </is>
       </c>
       <c r="C153" s="7" t="n"/>
@@ -2876,12 +2876,12 @@
     <row r="154" ht="15" customHeight="1" s="9">
       <c r="A154" s="7" t="inlineStr">
         <is>
-          <t>L1.6</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="B154" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ส่งอีเมลแจ้งผลการอนุมัติ</t>
+          <t xml:space="preserve">    สร้างใบแจ้งหนี้นักเรียน (Invoice Creation)</t>
         </is>
       </c>
       <c r="C154" s="7" t="n"/>
@@ -2890,12 +2890,12 @@
     <row r="155" ht="15" customHeight="1" s="9">
       <c r="A155" s="7" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L2.1</t>
         </is>
       </c>
       <c r="B155" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    สร้างใบแจ้งหนี้นักเรียน (Invoice Creation)</t>
+          <t xml:space="preserve">        ค้นหาและเลือกนักเรียน</t>
         </is>
       </c>
       <c r="C155" s="7" t="n"/>
@@ -2904,47 +2904,33 @@
     <row r="156" ht="105" customHeight="1" s="9">
       <c r="A156" s="7" t="inlineStr">
         <is>
-          <t>L2.1</t>
+          <t>L2.2</t>
         </is>
       </c>
       <c r="B156" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาและเลือกนักเรียน</t>
-        </is>
-      </c>
-      <c r="C156" s="7" t="n"/>
+          <t xml:space="preserve">        เลือกรายการค่าใช้จ่าย</t>
+        </is>
+      </c>
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>เลือกจากรายการที่มีอยู่ หรือสร้างรายการใหม่</t>
+        </is>
+      </c>
       <c r="D156" s="7" t="n"/>
     </row>
     <row r="157" ht="15" customHeight="1" s="9">
       <c r="A157" s="7" t="inlineStr">
         <is>
-          <t>L2.2</t>
+          <t>L2.3</t>
         </is>
       </c>
       <c r="B157" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เลือกรายการค่าใช้จ่าย</t>
+          <t xml:space="preserve">        คำนวณส่วนลดอัตโนมัติ 7 ประเภท</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
-        <is>
-          <t>เลือกจากรายการที่มีอยู่ หรือสร้างรายการใหม่</t>
-        </is>
-      </c>
-      <c r="D157" s="7" t="n"/>
-    </row>
-    <row r="158" ht="15" customHeight="1" s="9">
-      <c r="A158" s="7" t="inlineStr">
-        <is>
-          <t>L2.3</t>
-        </is>
-      </c>
-      <c r="B158" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        คำนวณส่วนลดอัตโนมัติ 7 ประเภท</t>
-        </is>
-      </c>
-      <c r="C158" s="7" t="inlineStr">
         <is>
           <t>1. Student Group
 2. Sibling
@@ -2955,17 +2941,31 @@
 7. Percentage</t>
         </is>
       </c>
+      <c r="D157" s="7" t="n"/>
+    </row>
+    <row r="158" ht="15" customHeight="1" s="9">
+      <c r="A158" s="7" t="inlineStr">
+        <is>
+          <t>L2.4</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        กำหนดวันครบกำหนดชำระ และหมายเหตุ</t>
+        </is>
+      </c>
+      <c r="C158" s="7" t="n"/>
       <c r="D158" s="7" t="n"/>
     </row>
     <row r="159" ht="15" customHeight="1" s="9">
       <c r="A159" s="7" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5</t>
         </is>
       </c>
       <c r="B159" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        กำหนดวันครบกำหนดชำระ และหมายเหตุ</t>
+          <t xml:space="preserve">        บันทึก Draft และ Submit เพื่ออนุมัติ</t>
         </is>
       </c>
       <c r="C159" s="7" t="n"/>
@@ -2974,12 +2974,12 @@
     <row r="160" ht="15" customHeight="1" s="9">
       <c r="A160" s="7" t="inlineStr">
         <is>
-          <t>L2.5</t>
+          <t>L2.6</t>
         </is>
       </c>
       <c r="B160" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        บันทึก Draft และ Submit เพื่ออนุมัติ</t>
+          <t xml:space="preserve">        สร้างและดาวน์โหลด PDF ใบแจ้งหนี้</t>
         </is>
       </c>
       <c r="C160" s="7" t="n"/>
@@ -2988,12 +2988,12 @@
     <row r="161" ht="15" customHeight="1" s="9">
       <c r="A161" s="7" t="inlineStr">
         <is>
-          <t>L2.6</t>
+          <t>L2.7</t>
         </is>
       </c>
       <c r="B161" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        สร้างและดาวน์โหลด PDF ใบแจ้งหนี้</t>
+          <t xml:space="preserve">        Export Interface File สำหรับระบบบัญชี</t>
         </is>
       </c>
       <c r="C161" s="7" t="n"/>
@@ -3002,12 +3002,12 @@
     <row r="162" ht="15" customHeight="1" s="9">
       <c r="A162" s="7" t="inlineStr">
         <is>
-          <t>L2.7</t>
+          <t>L2.8</t>
         </is>
       </c>
       <c r="B162" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Export Interface File สำหรับระบบบัญชี</t>
+          <t xml:space="preserve">        บันทึกและเรียกใช้ Template ใบแจ้งหนี้</t>
         </is>
       </c>
       <c r="C162" s="7" t="n"/>
@@ -3016,12 +3016,12 @@
     <row r="163" ht="15" customHeight="1" s="9">
       <c r="A163" s="7" t="inlineStr">
         <is>
-          <t>L2.8</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="B163" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        บันทึกและเรียกใช้ Template ใบแจ้งหนี้</t>
+          <t xml:space="preserve">    สร้างใบแจ้งหนี้ภายนอก (External Invoice Creation)</t>
         </is>
       </c>
       <c r="C163" s="7" t="n"/>
@@ -3030,12 +3030,12 @@
     <row r="164" ht="15" customHeight="1" s="9">
       <c r="A164" s="7" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L3.1</t>
         </is>
       </c>
       <c r="B164" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    สร้างใบแจ้งหนี้ภายนอก (External Invoice Creation)</t>
+          <t xml:space="preserve">        ระบุข้อมูลผู้รับ (ชื่อ, ที่อยู่, อีเมล)</t>
         </is>
       </c>
       <c r="C164" s="7" t="n"/>
@@ -3044,73 +3044,77 @@
     <row r="165" ht="18" customHeight="1" s="9">
       <c r="A165" s="7" t="inlineStr">
         <is>
-          <t>L3.1</t>
+          <t>L3.2</t>
         </is>
       </c>
       <c r="B165" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ระบุข้อมูลผู้รับ (ชื่อ, ที่อยู่, อีเมล)</t>
+          <t xml:space="preserve">        เลือกรายการ, คำนวณยอด, สร้าง PDF</t>
         </is>
       </c>
       <c r="C165" s="7" t="n"/>
       <c r="D165" s="7" t="n"/>
     </row>
     <row r="166" ht="15" customHeight="1" s="9">
-      <c r="A166" s="7" t="inlineStr">
-        <is>
-          <t>L3.2</t>
-        </is>
-      </c>
-      <c r="B166" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        เลือกรายการ, คำนวณยอด, สร้าง PDF</t>
-        </is>
-      </c>
-      <c r="C166" s="7" t="n"/>
-      <c r="D166" s="7" t="n"/>
+      <c r="A166" s="6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B166" s="6" t="inlineStr">
+        <is>
+          <t>ตั้งค่าระบบ (Settings &amp; Administration)</t>
+        </is>
+      </c>
+      <c r="C166" s="6" t="n"/>
+      <c r="D166" s="6" t="n"/>
     </row>
     <row r="167" ht="15" customHeight="1" s="9">
-      <c r="A167" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B167" s="6" t="inlineStr">
-        <is>
-          <t>ตั้งค่าระบบ (Settings &amp; Administration)</t>
-        </is>
-      </c>
-      <c r="C167" s="6" t="n"/>
-      <c r="D167" s="6" t="n"/>
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ตั้งค่าโรงเรียน (School Settings)</t>
+        </is>
+      </c>
+      <c r="C167" s="7" t="n"/>
+      <c r="D167" s="7" t="n"/>
     </row>
     <row r="168" ht="15" customHeight="1" s="9">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M1.1</t>
         </is>
       </c>
       <c r="B168" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ตั้งค่าโรงเรียน (School Settings)</t>
-        </is>
-      </c>
-      <c r="C168" s="7" t="n"/>
+          <t xml:space="preserve">        แก้ไขข้อมูลโรงเรียน</t>
+        </is>
+      </c>
+      <c r="C168" s="7" t="inlineStr">
+        <is>
+          <t>ฟิลด์: ชื่อ (EN/TH), ที่อยู่, เบอร์โทร, อีเมล, เว็บไซต์, Tax ID, โลโก้</t>
+        </is>
+      </c>
       <c r="D168" s="7" t="n"/>
     </row>
     <row r="169" ht="30" customHeight="1" s="9">
       <c r="A169" s="7" t="inlineStr">
         <is>
-          <t>M1.1</t>
+          <t>M1.2</t>
         </is>
       </c>
       <c r="B169" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        แก้ไขข้อมูลโรงเรียน</t>
+          <t xml:space="preserve">        ตั้งค่าบัญชีธนาคารสำหรับใบแจ้งหนี้</t>
         </is>
       </c>
       <c r="C169" s="7" t="inlineStr">
         <is>
-          <t>ฟิลด์: ชื่อ (EN/TH), ที่อยู่, เบอร์โทร, อีเมล, เว็บไซต์, Tax ID, โลโก้</t>
+          <t>ฟิลด์: ธนาคาร, ชื่อบัญชี, เลขบัญชี, สาขา, SWIFT Code</t>
         </is>
       </c>
       <c r="D169" s="7" t="n"/>
@@ -3118,17 +3122,18 @@
     <row r="170" ht="15" customHeight="1" s="9">
       <c r="A170" s="7" t="inlineStr">
         <is>
-          <t>M1.2</t>
+          <t>M1.3</t>
         </is>
       </c>
       <c r="B170" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ตั้งค่าบัญชีธนาคารสำหรับใบแจ้งหนี้</t>
+          <t xml:space="preserve">        Reset ข้อมูลระบบ (เลือกเฉพาะบางส่วน)</t>
         </is>
       </c>
       <c r="C170" s="7" t="inlineStr">
         <is>
-          <t>ฟิลด์: ธนาคาร, ชื่อบัญชี, เลขบัญชี, สาขา, SWIFT Code</t>
+          <t>คงไว้: users, activityLogs, authUser, app-language
+ลบ: ใบแจ้งหนี้, ค่าเทอม, ส่วนลด</t>
         </is>
       </c>
       <c r="D170" s="7" t="n"/>
@@ -3136,128 +3141,123 @@
     <row r="171" ht="15" customHeight="1" s="9">
       <c r="A171" s="7" t="inlineStr">
         <is>
-          <t>M1.3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="B171" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Reset ข้อมูลระบบ (เลือกเฉพาะบางส่วน)</t>
-        </is>
-      </c>
-      <c r="C171" s="7" t="inlineStr">
-        <is>
-          <t>คงไว้: users, activityLogs, authUser, app-language
-ลบ: ใบแจ้งหนี้, ค่าเทอม, ส่วนลด</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    ตั้งค่าบัญชีธนาคาร (Bank Settings)</t>
+        </is>
+      </c>
+      <c r="C171" s="7" t="n"/>
       <c r="D171" s="7" t="n"/>
     </row>
     <row r="172" ht="15" customHeight="1" s="9">
       <c r="A172" s="7" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M2.1</t>
         </is>
       </c>
       <c r="B172" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ตั้งค่าบัญชีธนาคาร (Bank Settings)</t>
-        </is>
-      </c>
-      <c r="C172" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ บัญชีธนาคาร</t>
+        </is>
+      </c>
+      <c r="C172" s="7" t="inlineStr">
+        <is>
+          <t>รองรับหลายบัญชี กำหนดบัญชีหลัก (Primary)</t>
+        </is>
+      </c>
       <c r="D172" s="7" t="n"/>
     </row>
     <row r="173" ht="30" customHeight="1" s="9">
       <c r="A173" s="7" t="inlineStr">
         <is>
-          <t>M2.1</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B173" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ บัญชีธนาคาร</t>
-        </is>
-      </c>
-      <c r="C173" s="7" t="inlineStr">
-        <is>
-          <t>รองรับหลายบัญชี กำหนดบัญชีหลัก (Primary)</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    ตั้งค่าเทอมเรียน (Term Settings)</t>
+        </is>
+      </c>
+      <c r="C173" s="7" t="n"/>
       <c r="D173" s="7" t="n"/>
     </row>
     <row r="174" ht="15" customHeight="1" s="9">
       <c r="A174" s="7" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M3.1</t>
         </is>
       </c>
       <c r="B174" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ตั้งค่าเทอมเรียน (Term Settings)</t>
-        </is>
-      </c>
-      <c r="C174" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข ปีการศึกษาและเทอม</t>
+        </is>
+      </c>
+      <c r="C174" s="7" t="inlineStr">
+        <is>
+          <t>กำหนด: วันเริ่ม-สิ้นสุดแต่ละเทอม
+ตรวจสอบ: วันที่ทับซ้อน, ปีต่อเนื่อง, สูงสุด 3 เทอม/ปี</t>
+        </is>
+      </c>
       <c r="D174" s="7" t="n"/>
     </row>
     <row r="175" ht="15" customHeight="1" s="9">
       <c r="A175" s="7" t="inlineStr">
         <is>
-          <t>M3.1</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B175" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข ปีการศึกษาและเทอม</t>
-        </is>
-      </c>
-      <c r="C175" s="7" t="inlineStr">
-        <is>
-          <t>กำหนด: วันเริ่ม-สิ้นสุดแต่ละเทอม
-ตรวจสอบ: วันที่ทับซ้อน, ปีต่อเนื่อง, สูงสุด 3 เทอม/ปี</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    จัดการผู้ใช้งาน (User Management)</t>
+        </is>
+      </c>
+      <c r="C175" s="7" t="n"/>
       <c r="D175" s="7" t="n"/>
     </row>
     <row r="176" ht="15" customHeight="1" s="9">
       <c r="A176" s="7" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M4.1</t>
         </is>
       </c>
       <c r="B176" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    จัดการผู้ใช้งาน (User Management)</t>
-        </is>
-      </c>
-      <c r="C176" s="7" t="n"/>
+          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ผู้ใช้งาน</t>
+        </is>
+      </c>
+      <c r="C176" s="7" t="inlineStr">
+        <is>
+          <t>ฟิลด์: Username, Email, ชื่อ-นามสกุล, Role, สถานะ</t>
+        </is>
+      </c>
       <c r="D176" s="7" t="n"/>
     </row>
     <row r="177" ht="15" customHeight="1" s="9">
       <c r="A177" s="7" t="inlineStr">
         <is>
-          <t>M4.1</t>
+          <t>M4.2</t>
         </is>
       </c>
       <c r="B177" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เพิ่ม / แก้ไข / ลบ ผู้ใช้งาน</t>
-        </is>
-      </c>
-      <c r="C177" s="7" t="inlineStr">
-        <is>
-          <t>ฟิลด์: Username, Email, ชื่อ-นามสกุล, Role, สถานะ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        กำหนด Role: Admin / Admin Accountant / Viewer / Approver</t>
+        </is>
+      </c>
+      <c r="C177" s="7" t="n"/>
       <c r="D177" s="7" t="n"/>
     </row>
     <row r="178" ht="15" customHeight="1" s="9">
       <c r="A178" s="7" t="inlineStr">
         <is>
-          <t>M4.2</t>
+          <t>M4.3</t>
         </is>
       </c>
       <c r="B178" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        กำหนด Role: Admin / Admin Accountant / Viewer / Approver</t>
+          <t xml:space="preserve">        ค้นหาตามชื่อ / Role / อีเมล และแบ่งหน้า</t>
         </is>
       </c>
       <c r="C178" s="7" t="n"/>
@@ -3266,12 +3266,12 @@
     <row r="179" ht="15" customHeight="1" s="9">
       <c r="A179" s="7" t="inlineStr">
         <is>
-          <t>M4.3</t>
+          <t>M4.4</t>
         </is>
       </c>
       <c r="B179" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาตามชื่อ / Role / อีเมล และแบ่งหน้า</t>
+          <t xml:space="preserve">        ส่งอีเมล Reset รหัสผ่าน</t>
         </is>
       </c>
       <c r="C179" s="7" t="n"/>
@@ -3280,12 +3280,12 @@
     <row r="180" ht="15" customHeight="1" s="9">
       <c r="A180" s="7" t="inlineStr">
         <is>
-          <t>M4.4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B180" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ส่งอีเมล Reset รหัสผ่าน</t>
+          <t xml:space="preserve">    บันทึกกิจกรรมระบบ (Activity Log)</t>
         </is>
       </c>
       <c r="C180" s="7" t="n"/>
@@ -3294,44 +3294,44 @@
     <row r="181" ht="15" customHeight="1" s="9">
       <c r="A181" s="7" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M5.1</t>
         </is>
       </c>
       <c r="B181" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    บันทึกกิจกรรมระบบ (Activity Log)</t>
-        </is>
-      </c>
-      <c r="C181" s="7" t="n"/>
+          <t xml:space="preserve">        ดูประวัติการดำเนินการทั้งหมด</t>
+        </is>
+      </c>
+      <c r="C181" s="7" t="inlineStr">
+        <is>
+          <t>บันทึก: ผู้ใช้, Action, Module, วัน-เวลา</t>
+        </is>
+      </c>
       <c r="D181" s="7" t="n"/>
     </row>
     <row r="182" ht="15" customHeight="1" s="9">
       <c r="A182" s="7" t="inlineStr">
         <is>
-          <t>M5.1</t>
+          <t>M5.2</t>
         </is>
       </c>
       <c r="B182" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ดูประวัติการดำเนินการทั้งหมด</t>
-        </is>
-      </c>
-      <c r="C182" s="7" t="inlineStr">
-        <is>
-          <t>บันทึก: ผู้ใช้, Action, Module, วัน-เวลา</t>
-        </is>
-      </c>
+          <t xml:space="preserve">        ค้นหาและกรองประวัติ และแบ่งหน้า</t>
+        </is>
+      </c>
+      <c r="C182" s="7" t="n"/>
       <c r="D182" s="7" t="n"/>
     </row>
     <row r="183" ht="15" customHeight="1" s="9">
       <c r="A183" s="7" t="inlineStr">
         <is>
-          <t>M5.2</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="B183" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ค้นหาและกรองประวัติ และแบ่งหน้า</t>
+          <t xml:space="preserve">    โปรไฟล์และการตั้งค่าผู้ใช้</t>
         </is>
       </c>
       <c r="C183" s="7" t="n"/>
@@ -3340,12 +3340,12 @@
     <row r="184" ht="15" customHeight="1" s="9">
       <c r="A184" s="7" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M6.1</t>
         </is>
       </c>
       <c r="B184" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    โปรไฟล์และการตั้งค่าผู้ใช้</t>
+          <t xml:space="preserve">        แก้ไขข้อมูลส่วนตัว และเปลี่ยนรหัสผ่าน</t>
         </is>
       </c>
       <c r="C184" s="7" t="n"/>
@@ -3354,12 +3354,12 @@
     <row r="185" ht="15" customHeight="1" s="9">
       <c r="A185" s="7" t="inlineStr">
         <is>
-          <t>M6.1</t>
+          <t>M6.2</t>
         </is>
       </c>
       <c r="B185" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        แก้ไขข้อมูลส่วนตัว และเปลี่ยนรหัสผ่าน</t>
+          <t xml:space="preserve">        เลือกภาษา: ไทย / อังกฤษ</t>
         </is>
       </c>
       <c r="C185" s="7" t="n"/>
@@ -3368,30 +3368,16 @@
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
         <is>
-          <t>M6.2</t>
+          <t>M6.3</t>
         </is>
       </c>
       <c r="B186" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        เลือกภาษา: ไทย / อังกฤษ</t>
+          <t xml:space="preserve">        ดูประวัติกิจกรรมส่วนตัว</t>
         </is>
       </c>
       <c r="C186" s="7" t="n"/>
       <c r="D186" s="7" t="n"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="7" t="inlineStr">
-        <is>
-          <t>M6.3</t>
-        </is>
-      </c>
-      <c r="B187" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ดูประวัติกิจกรรมส่วนตัว</t>
-        </is>
-      </c>
-      <c r="C187" s="7" t="n"/>
-      <c r="D187" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs: Update L2.3 discount types to 5 with correct description
- All types managed via Discount Management (% or Fixed Amount)
- Staff Child 100% excluded from invoice creation
- Duplicate discount per student not allowed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Feature_List_PaymentBackoffice_02032026.xlsx
+++ b/docs/Feature_List_PaymentBackoffice_02032026.xlsx
@@ -2927,18 +2927,20 @@
       </c>
       <c r="B157" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        คำนวณส่วนลดอัตโนมัติ 7 ประเภท</t>
+          <t xml:space="preserve">        คำนวณส่วนลดอัตโนมัติ 5 ประเภท</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>1. Student Group
+          <t>ทุกประเภทบริหารผ่าน Discount Management (Admin สร้างกลุ่ม + กำหนด % หรือ Fixed Amount)
+1. Student Group
 2. Sibling
 3. Staff Child
 4. Scholarship
 5. Early Bird
-6. Fixed Amount
-7. Percentage</t>
+หมายเหตุ:
+- Staff Child 100% → นักเรียนไม่แสดงในหน้าสร้าง Invoice
+- นักเรียนที่มี discount ประเภทนั้นอยู่แล้ว → ไม่สามารถเพิ่มซ้ำได้</t>
         </is>
       </c>
       <c r="D157" s="7" t="n"/>

</xml_diff>

<commit_message>
feat: Add template dialogs, pagination, cancel confirmation, and xlsx docs
- Add standalone EditTemplateDialog to InvoiceManagement (fix nested dialog issue)
- Add Receipt Template button to ReceiptPageUpdated and ReceiptManagementFlow
- Add cancel confirmation dialog to DebtReminderSettings before cancelling scheduled email
- Add pagination to ReceiptManagementFlow and other list pages
- Fill 57 empty Description cells in Feature_List xlsx documentation
- Table alignment standardization across multiple components

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Feature_List_PaymentBackoffice_02032026.xlsx
+++ b/docs/Feature_List_PaymentBackoffice_02032026.xlsx
@@ -689,8 +689,11 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Approver เข้าได้เฉพาะ Approval Queue, User Profile, Settings, Activity
-หน้าอื่นถูก redirect กลับ</t>
+          <t>ระบบควบคุมการเข้าถึงตาม Role ของผู้ใช้
+- Super Admin: เข้าถึงได้ทุกหน้าโดยไม่มีข้อจำกัด
+- AdminAccountant: เข้าถึงได้ทุกหน้า ยกเว้น User Management
+- Viewer: เข้าถึงได้ทุกหน้า แต่เป็น Read-only ไม่สามารถแก้ไขข้อมูลได้
+- Approver: เข้าได้เฉพาะ Approval Queue, User Profile, Settings และ Activity หากพยายามเข้าหน้าอื่น ระบบจะ redirect กลับไปยัง Approval Queue โดยอัตโนมัติ</t>
         </is>
       </c>
       <c r="D12" s="7" t="n"/>
@@ -929,7 +932,15 @@
           <t xml:space="preserve">        ติดตามสถานะ: Draft / Scheduled / Sent / Cancelled</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n"/>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>ระบบแสดงสถานะของการแจ้งเตือนแต่ละรายการ
+- Draft: ยังไม่ได้กำหนดเวลาส่ง สามารถแก้ไขได้
+- Scheduled: กำหนดเวลาส่งแล้ว ระบบล็อกการแก้ไข
+- Sent: ส่ง Email เรียบร้อยแล้ว บันทึกวันเวลาไว้ในประวัติ
+- Cancelled: ยกเลิก Schedule แล้ว สถานะกลับเป็น Draft</t>
+        </is>
+      </c>
       <c r="D26" s="7" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="9">
@@ -993,7 +1004,11 @@
           <t xml:space="preserve">        บันทึกและ Reset template กลับค่าเริ่มต้น</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>ผู้ใช้สามารถบันทึก Template ที่แก้ไขแล้ว หรือ Reset กลับค่าเริ่มต้น (Default Template) ได้ตลอดเวลา</t>
+        </is>
+      </c>
       <c r="D30" s="7" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="9">
@@ -1039,7 +1054,14 @@
           <t xml:space="preserve">        ค้นหาตามผู้รับ / ประเภท / หัวข้ออีเมล</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n"/>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>รองรับการค้นหาจากหลายเงื่อนไขร่วมกัน
+- ผู้รับ: ชื่อผู้ปกครองหรือ Email
+- ประเภท: Invoice, Receipt, Reminder
+- หัวข้ออีเมล: Subject ของ Email ที่ส่งออกไป</t>
+        </is>
+      </c>
       <c r="D33" s="7" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="9">
@@ -1053,7 +1075,11 @@
           <t xml:space="preserve">        Export ประวัติการส่งเป็นไฟล์ Excel</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n"/>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Export ประวัติการส่ง Email ทั้งหมดหรือที่กรองแล้วออกเป็นไฟล์ Excel (.xlsx)</t>
+        </is>
+      </c>
       <c r="D34" s="7" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="9">
@@ -1099,7 +1125,15 @@
           <t xml:space="preserve">        กรองตามวันที่ / สถานะ / นักเรียน / ยอดเงิน</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n"/>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>รองรับการกรองหลายเงื่อนไขพร้อมกัน
+- วันที่: ช่วงวันที่ชำระ
+- สถานะ: Paid, Pending, Failed
+- นักเรียน: ชื่อหรือรหัสนักเรียน
+- ยอดเงิน: ระบุช่วงขั้นต่ำ-สูงสุด</t>
+        </is>
+      </c>
       <c r="D37" s="7" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="9">
@@ -1113,7 +1147,11 @@
           <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n"/>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>รองรับการจัดเรียงข้อมูลโดยกดที่หัวคอลัมน์ (ascending/descending) และแบ่งหน้าแสดงผลพร้อมตั้งค่าจำนวนรายการต่อหน้า</t>
+        </is>
+      </c>
       <c r="D38" s="7" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="9">
@@ -1127,7 +1165,11 @@
           <t xml:space="preserve">        Export ข้อมูลเป็นไฟล์ Excel</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n"/>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Export รายการชำระเงินทั้งหมดหรือที่กรองแล้วออกเป็นไฟล์ Excel (.xlsx)</t>
+        </is>
+      </c>
       <c r="D39" s="7" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="9">
@@ -1206,7 +1248,11 @@
           <t xml:space="preserve">        เลือกแสดงข้อมูลตามปีการศึกษา</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n"/>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>เลือกดูข้อมูลอัตราค่าเทอมตามปีการศึกษาที่ต้องการได้จาก Dropdown</t>
+        </is>
+      </c>
       <c r="D44" s="7" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="9">
@@ -1252,7 +1298,11 @@
           <t xml:space="preserve">        เปิด / ปิด การใช้งานกลุ่มส่วนลด</t>
         </is>
       </c>
-      <c r="C47" s="7" t="n"/>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>สามารถเปิดหรือปิดการใช้งานกลุ่มส่วนลดได้โดยไม่ต้องลบข้อมูล เพื่อนำกลับมาใช้ในภายหลัง</t>
+        </is>
+      </c>
       <c r="D47" s="7" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="9">
@@ -1312,7 +1362,11 @@
           <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C51" s="7" t="n"/>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>รองรับการจัดเรียงข้อมูลโดยกดที่หัวคอลัมน์ (ascending/descending) และแบ่งหน้าแสดงผลพร้อมตั้งค่าจำนวนรายการต่อหน้า</t>
+        </is>
+      </c>
       <c r="D51" s="7" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="9">
@@ -1362,7 +1416,14 @@
           <t xml:space="preserve">        Export ใบแจ้งหนี้เป็น Excel / ZIP / PDF</t>
         </is>
       </c>
-      <c r="C54" s="7" t="n"/>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Export ใบแจ้งหนี้ในรูปแบบที่ต้องการ
+- Excel (.xlsx): ข้อมูลสรุปทุกใบ
+- ZIP: รวม PDF ทุกใบในไฟล์เดียว
+- PDF: รายใบ</t>
+        </is>
+      </c>
       <c r="D54" s="7" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="9">
@@ -1376,7 +1437,11 @@
           <t xml:space="preserve">        ส่งใบแจ้งหนี้ทางอีเมล พร้อมบันทึก Log</t>
         </is>
       </c>
-      <c r="C55" s="7" t="n"/>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>ส่งใบแจ้งหนี้ไปยัง Email ของผู้ปกครอง พร้อมบันทึก Log วัน-เวลา และสถานะการส่ง (Sent/Failed)</t>
+        </is>
+      </c>
       <c r="D55" s="7" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="9">
@@ -1472,7 +1537,11 @@
           <t xml:space="preserve">        ค้นหาตามรหัส / ชื่อ / ชั้นเรียน และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C61" s="7" t="n"/>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหารายการจากรหัส, ชื่อ, หรือชั้นเรียน พร้อมแบ่งหน้าแสดงผลและตั้งค่าจำนวนรายการต่อหน้า</t>
+        </is>
+      </c>
       <c r="D61" s="7" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="9">
@@ -1504,7 +1573,11 @@
           <t xml:space="preserve">        เปิด / ปิด การใช้งานรายการ (Active/Inactive)</t>
         </is>
       </c>
-      <c r="C63" s="7" t="n"/>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Toggle เปิด/ปิดการใช้งานรายการค่าใช้จ่ายได้โดยไม่ต้องลบ รายการที่ปิดจะไม่แสดงในขั้นตอนสร้างใบแจ้งหนี้</t>
+        </is>
+      </c>
       <c r="D63" s="7" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="9">
@@ -1582,7 +1655,11 @@
           <t xml:space="preserve">        สร้าง PDF ใบเสร็จรับเงิน</t>
         </is>
       </c>
-      <c r="C68" s="7" t="n"/>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>สร้างไฟล์ PDF ใบเสร็จรับเงินที่รวมข้อมูลโรงเรียน รายการชำระ และข้อมูลผู้ชำระ สามารถดาวน์โหลดหรือพิมพ์ได้</t>
+        </is>
+      </c>
       <c r="D68" s="7" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="9">
@@ -1596,7 +1673,11 @@
           <t xml:space="preserve">        นำเข้าและ Export ข้อมูลใบเสร็จ</t>
         </is>
       </c>
-      <c r="C69" s="7" t="n"/>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>นำเข้าข้อมูลใบเสร็จจาก Excel และ Export ข้อมูลใบเสร็จทั้งหมดออกเป็น Excel (.xlsx)</t>
+        </is>
+      </c>
       <c r="D69" s="7" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="9">
@@ -1643,7 +1724,11 @@
           <t xml:space="preserve">        ค้นหาตามเลขที่ / ชื่อนักเรียน / สถานะ และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C72" s="7" t="n"/>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหาตามเลขที่ใบลดหนี้, ชื่อนักเรียน หรือสถานะ พร้อมแบ่งหน้าแสดงผล</t>
+        </is>
+      </c>
       <c r="D72" s="7" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="9">
@@ -1657,7 +1742,11 @@
           <t xml:space="preserve">        นำเข้าและ Export ข้อมูลใบลดหนี้เป็น Excel</t>
         </is>
       </c>
-      <c r="C73" s="7" t="n"/>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>นำเข้าข้อมูลใบลดหนี้จาก Excel และ Export ข้อมูลออกเป็นไฟล์ Excel (.xlsx)</t>
+        </is>
+      </c>
       <c r="D73" s="7" t="n"/>
     </row>
     <row r="74" ht="18" customHeight="1" s="9">
@@ -1763,7 +1852,11 @@
           <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
-      <c r="C80" s="7" t="n"/>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์เหมือนกับ Tuition Receipt: ดูรายการ, Bulk Actions, Export Excel, สร้าง PDF ใบเสร็จ หมวดหมู่: ECA</t>
+        </is>
+      </c>
       <c r="D80" s="7" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1" s="9">
@@ -1791,7 +1884,11 @@
           <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด ECA</t>
         </is>
       </c>
-      <c r="C82" s="7" t="n"/>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>เพิ่ม/แก้ไข/ลบ กลุ่มส่วนลดเฉพาะหมวด ECA กำหนดประเภทส่วนลดแบบ % หรือ Fixed Amount และเปิด/ปิดการใช้งาน</t>
+        </is>
+      </c>
       <c r="D82" s="7" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1" s="9">
@@ -1865,7 +1962,11 @@
           <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
         </is>
       </c>
-      <c r="C87" s="7" t="n"/>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์เหมือนกับ Tuition Items: CRUD, นำเข้าจาก Excel, Export หมวดหมู่: trip</t>
+        </is>
+      </c>
       <c r="D87" s="7" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="9">
@@ -1893,7 +1994,11 @@
           <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
-      <c r="C89" s="7" t="n"/>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์เหมือนกับ Tuition Receipt: ดูรายการ, Bulk Actions, Export Excel, สร้าง PDF ใบเสร็จ หมวดหมู่: trip</t>
+        </is>
+      </c>
       <c r="D89" s="7" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1" s="9">
@@ -1921,7 +2026,11 @@
           <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Trip</t>
         </is>
       </c>
-      <c r="C91" s="7" t="n"/>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>เพิ่ม/แก้ไข/ลบ กลุ่มส่วนลดเฉพาะหมวด Trip กำหนดประเภทส่วนลดแบบ % หรือ Fixed Amount และเปิด/ปิดการใช้งาน</t>
+        </is>
+      </c>
       <c r="D91" s="7" t="n"/>
     </row>
     <row r="92" ht="18" customHeight="1" s="9">
@@ -1995,7 +2104,11 @@
           <t xml:space="preserve">        CRUD, Import, Export — เหมือน Tuition Items</t>
         </is>
       </c>
-      <c r="C96" s="7" t="n"/>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์เหมือนกับ Tuition Items: CRUD, นำเข้าจาก Excel, Export หมวดหมู่: exam</t>
+        </is>
+      </c>
       <c r="D96" s="7" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1" s="9">
@@ -2023,7 +2136,11 @@
           <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
-      <c r="C98" s="7" t="n"/>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์เหมือนกับ Tuition Receipt: ดูรายการ, Bulk Actions, Export Excel, สร้าง PDF ใบเสร็จ หมวดหมู่: exam</t>
+        </is>
+      </c>
       <c r="D98" s="7" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="9">
@@ -2051,7 +2168,11 @@
           <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Exam</t>
         </is>
       </c>
-      <c r="C100" s="7" t="n"/>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>เพิ่ม/แก้ไข/ลบ กลุ่มส่วนลดเฉพาะหมวด Exam กำหนดประเภทส่วนลดแบบ % หรือ Fixed Amount และเปิด/ปิดการใช้งาน</t>
+        </is>
+      </c>
       <c r="D100" s="7" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1" s="9">
@@ -2157,7 +2278,11 @@
           <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
-      <c r="C107" s="7" t="n"/>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์เหมือนกับ Tuition Receipt: ดูรายการ, Bulk Actions, Export Excel, สร้าง PDF ใบเสร็จ หมวดหมู่: bus</t>
+        </is>
+      </c>
       <c r="D107" s="7" t="n"/>
     </row>
     <row r="108" ht="15" customHeight="1" s="9">
@@ -2185,7 +2310,11 @@
           <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด Bus</t>
         </is>
       </c>
-      <c r="C109" s="7" t="n"/>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>เพิ่ม/แก้ไข/ลบ กลุ่มส่วนลดเฉพาะหมวด Bus กำหนดประเภทส่วนลดแบบ % หรือ Fixed Amount และเปิด/ปิดการใช้งาน</t>
+        </is>
+      </c>
       <c r="D109" s="7" t="n"/>
     </row>
     <row r="110" ht="18" customHeight="1" s="9">
@@ -2296,7 +2425,11 @@
           <t xml:space="preserve">        ค้นหาลูกค้า</t>
         </is>
       </c>
-      <c r="C116" s="7" t="n"/>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหาลูกค้าจากชื่อบริษัท/บุคคล, ชื่อผู้ติดต่อ หรือที่อยู่ พร้อมแบ่งหน้าแสดงผล</t>
+        </is>
+      </c>
       <c r="D116" s="7" t="n"/>
     </row>
     <row r="117" ht="30" customHeight="1" s="9">
@@ -2393,7 +2526,11 @@
           <t xml:space="preserve">        ดู, Bulk, Export, PDF — เหมือน Tuition Receipt</t>
         </is>
       </c>
-      <c r="C122" s="7" t="n"/>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์เหมือนกับ Tuition Receipt: ดูรายการ, Bulk Actions, Export Excel, สร้าง PDF ใบเสร็จ หมวดหมู่: external</t>
+        </is>
+      </c>
       <c r="D122" s="7" t="n"/>
     </row>
     <row r="123" ht="15" customHeight="1" s="9">
@@ -2421,7 +2558,11 @@
           <t xml:space="preserve">        CRUD กลุ่มส่วนลดเฉพาะหมวด External</t>
         </is>
       </c>
-      <c r="C124" s="7" t="n"/>
+      <c r="C124" s="7" t="inlineStr">
+        <is>
+          <t>เพิ่ม/แก้ไข/ลบ กลุ่มส่วนลดเฉพาะหมวด External กำหนดประเภทส่วนลดแบบ % หรือ Fixed Amount และเปิด/ปิดการใช้งาน</t>
+        </is>
+      </c>
       <c r="D124" s="7" t="n"/>
     </row>
     <row r="125" ht="18" customHeight="1" s="9">
@@ -2481,7 +2622,11 @@
           <t xml:space="preserve">        ค้นหาตามชื่อ / รหัส และกรองตามสถานะ / ชั้น / ปีการศึกษา / เทอม</t>
         </is>
       </c>
-      <c r="C128" s="7" t="n"/>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหาตามชื่อหรือรหัสนักเรียน และกรองตามสถานะ (Active/Inactive), ชั้นเรียน, ปีการศึกษา หรือเทอม</t>
+        </is>
+      </c>
       <c r="D128" s="7" t="n"/>
     </row>
     <row r="129" ht="15" customHeight="1" s="9">
@@ -2495,7 +2640,11 @@
           <t xml:space="preserve">        จัดเรียงข้อมูลตามคอลัมน์ และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C129" s="7" t="n"/>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>รองรับการจัดเรียงข้อมูลโดยกดที่หัวคอลัมน์ (ascending/descending) และแบ่งหน้าแสดงผลพร้อมตั้งค่าจำนวนรายการต่อหน้า</t>
+        </is>
+      </c>
       <c r="D129" s="7" t="n"/>
     </row>
     <row r="130" ht="30" customHeight="1" s="9">
@@ -2597,7 +2746,11 @@
           <t xml:space="preserve">        ค้นหาและกรองข้อมูลครอบครัว และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C135" s="7" t="n"/>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหาครอบครัวจาก Family Code หรือชื่อครอบครัว และกรองตามเงื่อนไข พร้อมแบ่งหน้าแสดงผล</t>
+        </is>
+      </c>
       <c r="D135" s="7" t="n"/>
     </row>
     <row r="136" ht="18" customHeight="1" s="9">
@@ -2611,7 +2764,11 @@
           <t xml:space="preserve">        Export ข้อมูลครอบครัวเป็น Excel</t>
         </is>
       </c>
-      <c r="C136" s="7" t="n"/>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
+          <t>Export ข้อมูลครอบครัวทั้งหมดออกเป็นไฟล์ Excel (.xlsx)</t>
+        </is>
+      </c>
       <c r="D136" s="7" t="n"/>
     </row>
     <row r="137" ht="15" customHeight="1" s="9">
@@ -2671,7 +2828,11 @@
           <t xml:space="preserve">        ติดตามสถานะ: Active / Ended / Scheduled [ถูกลบออกจากระบบ]</t>
         </is>
       </c>
-      <c r="C140" s="7" t="n"/>
+      <c r="C140" s="7" t="inlineStr">
+        <is>
+          <t>ฟีเจอร์นี้ถูกลบออกจากระบบแล้ว ไม่มีการแสดงผลในระบบปัจจุบัน</t>
+        </is>
+      </c>
       <c r="D140" s="7" t="n"/>
     </row>
     <row r="141" ht="15" customHeight="1" s="9">
@@ -2717,7 +2878,11 @@
           <t xml:space="preserve">        กรองตามสถานะและปีการศึกษา</t>
         </is>
       </c>
-      <c r="C143" s="7" t="n"/>
+      <c r="C143" s="7" t="inlineStr">
+        <is>
+          <t>กรองรายชื่อนักเรียนที่มีสิทธิ์ยกเว้นค่าเทอมตามสถานะ (Active/Inactive) และปีการศึกษา</t>
+        </is>
+      </c>
       <c r="D143" s="7" t="n"/>
     </row>
     <row r="144" ht="15" customHeight="1" s="9">
@@ -2828,7 +2993,11 @@
           <t xml:space="preserve">        กรองตามสถานะ / วันที่ / ชื่อนักเรียน และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C150" s="7" t="n"/>
+      <c r="C150" s="7" t="inlineStr">
+        <is>
+          <t>กรองรายการใบแจ้งหนี้ตามสถานะ (Wait/Approved/Rejected), ช่วงวันที่ หรือชื่อนักเรียน พร้อมแบ่งหน้าแสดงผล</t>
+        </is>
+      </c>
       <c r="D150" s="7" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1" s="9">
@@ -2842,7 +3011,11 @@
           <t xml:space="preserve">        ดำเนินการหลายรายการพร้อมกัน (Bulk Approve)</t>
         </is>
       </c>
-      <c r="C151" s="7" t="n"/>
+      <c r="C151" s="7" t="inlineStr">
+        <is>
+          <t>เลือกหลายรายการพร้อมกันและดำเนินการ Approve หรือ Reject ทีเดียว เพื่อเพิ่มประสิทธิภาพการทำงาน</t>
+        </is>
+      </c>
       <c r="D151" s="7" t="n"/>
     </row>
     <row r="152" ht="15" customHeight="1" s="9">
@@ -2856,7 +3029,11 @@
           <t xml:space="preserve">        Export ใบแจ้งหนี้เป็น Excel / PDF</t>
         </is>
       </c>
-      <c r="C152" s="7" t="n"/>
+      <c r="C152" s="7" t="inlineStr">
+        <is>
+          <t>Export ใบแจ้งหนี้ที่เลือกออกเป็น Excel (.xlsx) หรือ PDF</t>
+        </is>
+      </c>
       <c r="D152" s="7" t="n"/>
     </row>
     <row r="153" ht="15" customHeight="1" s="9">
@@ -2870,7 +3047,11 @@
           <t xml:space="preserve">        ส่งอีเมลแจ้งผลการอนุมัติ</t>
         </is>
       </c>
-      <c r="C153" s="7" t="n"/>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>ส่ง Email แจ้งผลการอนุมัติหรือปฏิเสธไปยังผู้ปกครองหลังจากดำเนินการเรียบร้อยแล้ว</t>
+        </is>
+      </c>
       <c r="D153" s="7" t="n"/>
     </row>
     <row r="154" ht="15" customHeight="1" s="9">
@@ -2898,7 +3079,11 @@
           <t xml:space="preserve">        ค้นหาและเลือกนักเรียน</t>
         </is>
       </c>
-      <c r="C155" s="7" t="n"/>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหานักเรียนจากชื่อหรือรหัส กรองตามชั้นเรียนหรือปีการศึกษา เพื่อเลือกผู้รับใบแจ้งหนี้</t>
+        </is>
+      </c>
       <c r="D155" s="7" t="n"/>
     </row>
     <row r="156" ht="105" customHeight="1" s="9">
@@ -2956,7 +3141,11 @@
           <t xml:space="preserve">        กำหนดวันครบกำหนดชำระ และหมายเหตุ</t>
         </is>
       </c>
-      <c r="C158" s="7" t="n"/>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>กำหนดวันที่ครบกำหนดชำระเงิน (Due Date) และเพิ่มหมายเหตุเพิ่มเติมในใบแจ้งหนี้ได้</t>
+        </is>
+      </c>
       <c r="D158" s="7" t="n"/>
     </row>
     <row r="159" ht="15" customHeight="1" s="9">
@@ -2970,7 +3159,11 @@
           <t xml:space="preserve">        บันทึก Draft และ Submit เพื่ออนุมัติ</t>
         </is>
       </c>
-      <c r="C159" s="7" t="n"/>
+      <c r="C159" s="7" t="inlineStr">
+        <is>
+          <t>บันทึกใบแจ้งหนี้เป็น Draft เพื่อแก้ไขภายหลัง หรือ Submit ส่งเข้าคิวเพื่อรออนุมัติ</t>
+        </is>
+      </c>
       <c r="D159" s="7" t="n"/>
     </row>
     <row r="160" ht="15" customHeight="1" s="9">
@@ -2984,7 +3177,11 @@
           <t xml:space="preserve">        สร้างและดาวน์โหลด PDF ใบแจ้งหนี้</t>
         </is>
       </c>
-      <c r="C160" s="7" t="n"/>
+      <c r="C160" s="7" t="inlineStr">
+        <is>
+          <t>สร้างและดาวน์โหลดไฟล์ PDF ใบแจ้งหนี้ที่รวมข้อมูลโรงเรียน รายการค่าใช้จ่าย ส่วนลด และบัญชีธนาคาร</t>
+        </is>
+      </c>
       <c r="D160" s="7" t="n"/>
     </row>
     <row r="161" ht="15" customHeight="1" s="9">
@@ -2998,7 +3195,11 @@
           <t xml:space="preserve">        Export Interface File สำหรับระบบบัญชี</t>
         </is>
       </c>
-      <c r="C161" s="7" t="n"/>
+      <c r="C161" s="7" t="inlineStr">
+        <is>
+          <t>Export Interface File ในรูปแบบ Excel สำหรับเชื่อมต่อและนำเข้าข้อมูลเข้าระบบบัญชีภายนอก</t>
+        </is>
+      </c>
       <c r="D161" s="7" t="n"/>
     </row>
     <row r="162" ht="15" customHeight="1" s="9">
@@ -3012,7 +3213,11 @@
           <t xml:space="preserve">        บันทึกและเรียกใช้ Template ใบแจ้งหนี้</t>
         </is>
       </c>
-      <c r="C162" s="7" t="n"/>
+      <c r="C162" s="7" t="inlineStr">
+        <is>
+          <t>บันทึก Email Template สำหรับส่งใบแจ้งหนี้ และเรียกใช้ Template ที่บันทึกไว้เมื่อต้องการส่ง Email</t>
+        </is>
+      </c>
       <c r="D162" s="7" t="n"/>
     </row>
     <row r="163" ht="15" customHeight="1" s="9">
@@ -3040,7 +3245,11 @@
           <t xml:space="preserve">        ระบุข้อมูลผู้รับ (ชื่อ, ที่อยู่, อีเมล)</t>
         </is>
       </c>
-      <c r="C164" s="7" t="n"/>
+      <c r="C164" s="7" t="inlineStr">
+        <is>
+          <t>กรอกข้อมูลผู้รับใบแจ้งหนี้ภายนอก ได้แก่ ชื่อบุคคล/บริษัท, ที่อยู่ และ Email สำหรับจัดส่งเอกสาร</t>
+        </is>
+      </c>
       <c r="D164" s="7" t="n"/>
     </row>
     <row r="165" ht="18" customHeight="1" s="9">
@@ -3054,7 +3263,11 @@
           <t xml:space="preserve">        เลือกรายการ, คำนวณยอด, สร้าง PDF</t>
         </is>
       </c>
-      <c r="C165" s="7" t="n"/>
+      <c r="C165" s="7" t="inlineStr">
+        <is>
+          <t>เลือกรายการค่าใช้จ่าย คำนวณยอดรวมอัตโนมัติ และสร้างไฟล์ PDF ใบแจ้งหนี้สำหรับลูกค้าภายนอก</t>
+        </is>
+      </c>
       <c r="D165" s="7" t="n"/>
     </row>
     <row r="166" ht="15" customHeight="1" s="9">
@@ -3248,7 +3461,15 @@
           <t xml:space="preserve">        กำหนด Role: Admin / Admin Accountant / Viewer / Approver</t>
         </is>
       </c>
-      <c r="C177" s="7" t="n"/>
+      <c r="C177" s="7" t="inlineStr">
+        <is>
+          <t>กำหนด Role ให้กับผู้ใช้งาน
+- Admin: สิทธิ์เต็มทุกหน้า
+- Admin Accountant: สิทธิ์ทุกหน้า ยกเว้น User Management
+- Viewer: Read-only ทุกหน้า
+- Approver: เข้าได้เฉพาะ Approval Queue, Profile, Settings, Activity</t>
+        </is>
+      </c>
       <c r="D177" s="7" t="n"/>
     </row>
     <row r="178" ht="15" customHeight="1" s="9">
@@ -3262,7 +3483,11 @@
           <t xml:space="preserve">        ค้นหาตามชื่อ / Role / อีเมล และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C178" s="7" t="n"/>
+      <c r="C178" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหาผู้ใช้งานจากชื่อ, Role หรือ Email พร้อมแบ่งหน้าแสดงผล</t>
+        </is>
+      </c>
       <c r="D178" s="7" t="n"/>
     </row>
     <row r="179" ht="15" customHeight="1" s="9">
@@ -3276,7 +3501,11 @@
           <t xml:space="preserve">        ส่งอีเมล Reset รหัสผ่าน</t>
         </is>
       </c>
-      <c r="C179" s="7" t="n"/>
+      <c r="C179" s="7" t="inlineStr">
+        <is>
+          <t>ส่ง Email ไปยังผู้ใช้งานเพื่อให้ดำเนินการ Reset รหัสผ่านด้วยตนเอง</t>
+        </is>
+      </c>
       <c r="D179" s="7" t="n"/>
     </row>
     <row r="180" ht="15" customHeight="1" s="9">
@@ -3322,7 +3551,11 @@
           <t xml:space="preserve">        ค้นหาและกรองประวัติ และแบ่งหน้า</t>
         </is>
       </c>
-      <c r="C182" s="7" t="n"/>
+      <c r="C182" s="7" t="inlineStr">
+        <is>
+          <t>ค้นหาและกรองประวัติกิจกรรมตามผู้ใช้, Action, Module หรือช่วงวันที่ พร้อมแบ่งหน้าแสดงผล</t>
+        </is>
+      </c>
       <c r="D182" s="7" t="n"/>
     </row>
     <row r="183" ht="15" customHeight="1" s="9">
@@ -3350,7 +3583,11 @@
           <t xml:space="preserve">        แก้ไขข้อมูลส่วนตัว และเปลี่ยนรหัสผ่าน</t>
         </is>
       </c>
-      <c r="C184" s="7" t="n"/>
+      <c r="C184" s="7" t="inlineStr">
+        <is>
+          <t>แก้ไขข้อมูลส่วนตัว เช่น ชื่อ, Email และเปลี่ยนรหัสผ่านได้จากหน้า Profile</t>
+        </is>
+      </c>
       <c r="D184" s="7" t="n"/>
     </row>
     <row r="185" ht="15" customHeight="1" s="9">
@@ -3364,7 +3601,11 @@
           <t xml:space="preserve">        เลือกภาษา: ไทย / อังกฤษ</t>
         </is>
       </c>
-      <c r="C185" s="7" t="n"/>
+      <c r="C185" s="7" t="inlineStr">
+        <is>
+          <t>เปลี่ยนภาษาที่แสดงผลในระบบ รองรับ 2 ภาษา: ไทย และ อังกฤษ การตั้งค่าจะถูกบันทึกไว้สำหรับผู้ใช้คนนั้น</t>
+        </is>
+      </c>
       <c r="D185" s="7" t="n"/>
     </row>
     <row r="186">
@@ -3378,7 +3619,11 @@
           <t xml:space="preserve">        ดูประวัติกิจกรรมส่วนตัว</t>
         </is>
       </c>
-      <c r="C186" s="7" t="n"/>
+      <c r="C186" s="7" t="inlineStr">
+        <is>
+          <t>ดูประวัติการดำเนินการของตนเองในระบบ เช่น การ Login, การสร้าง/แก้ไขข้อมูล</t>
+        </is>
+      </c>
       <c r="D186" s="7" t="n"/>
     </row>
   </sheetData>

</xml_diff>